<commit_message>
fix: corregir bracket R32 para evitar equipos duplicados
Los 8 mejores terceros se enfrentan entre sí (4 partidos) en lugar de
contra primeros ya incluidos en el bracket de 12 partidos.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/excel/Mundial_2026_Predicciones.xlsx
+++ b/results/excel/Mundial_2026_Predicciones.xlsx
@@ -5834,16 +5834,16 @@
         <v>1771</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.4628</v>
+        <v>0.459</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.2934</v>
+        <v>0.3006</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>0.1602</v>
+        <v>0.1642</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>0.08360000000000001</v>
+        <v>0.07619999999999993</v>
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
@@ -5862,16 +5862,16 @@
         <v>1746</v>
       </c>
       <c r="N5" s="19" t="n">
-        <v>0.5018</v>
+        <v>0.4804</v>
       </c>
       <c r="O5" s="19" t="n">
-        <v>0.2836</v>
+        <v>0.294</v>
       </c>
       <c r="P5" s="19" t="n">
-        <v>0.1476</v>
+        <v>0.1494</v>
       </c>
       <c r="Q5" s="19" t="n">
-        <v>0.06699999999999995</v>
+        <v>0.07620000000000007</v>
       </c>
       <c r="R5" s="17" t="inlineStr">
         <is>
@@ -5890,16 +5890,16 @@
         <v>1734</v>
       </c>
       <c r="X5" s="19" t="n">
-        <v>0.2756</v>
+        <v>0.2898</v>
       </c>
       <c r="Y5" s="19" t="n">
-        <v>0.2764</v>
+        <v>0.2746</v>
       </c>
       <c r="Z5" s="19" t="n">
-        <v>0.2284</v>
+        <v>0.2244</v>
       </c>
       <c r="AA5" s="19" t="n">
-        <v>0.2196</v>
+        <v>0.2111999999999999</v>
       </c>
       <c r="AB5" s="17" t="inlineStr">
         <is>
@@ -5918,16 +5918,16 @@
         <v>1838</v>
       </c>
       <c r="AH5" s="19" t="n">
-        <v>0.4552</v>
+        <v>0.456</v>
       </c>
       <c r="AI5" s="19" t="n">
-        <v>0.3454</v>
+        <v>0.3498</v>
       </c>
       <c r="AJ5" s="19" t="n">
-        <v>0.1522</v>
+        <v>0.1472</v>
       </c>
       <c r="AK5" s="19" t="n">
-        <v>0.04719999999999996</v>
+        <v>0.04700000000000004</v>
       </c>
       <c r="AL5" s="17" t="inlineStr">
         <is>
@@ -5948,16 +5948,16 @@
         <v>1725</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>0.3288</v>
+        <v>0.3272</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>0.3304</v>
+        <v>0.3258</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>0.2112</v>
+        <v>0.2242</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>0.1296</v>
+        <v>0.1228000000000001</v>
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
@@ -5976,16 +5976,16 @@
         <v>1685</v>
       </c>
       <c r="N6" s="22" t="n">
-        <v>0.306</v>
+        <v>0.328</v>
       </c>
       <c r="O6" s="22" t="n">
-        <v>0.3514</v>
+        <v>0.3368</v>
       </c>
       <c r="P6" s="22" t="n">
-        <v>0.2152</v>
+        <v>0.2184</v>
       </c>
       <c r="Q6" s="22" t="n">
-        <v>0.1274</v>
+        <v>0.1167999999999999</v>
       </c>
       <c r="R6" s="20" t="inlineStr">
         <is>
@@ -6007,13 +6007,13 @@
         <v>0.2738</v>
       </c>
       <c r="Y6" s="22" t="n">
-        <v>0.2634</v>
+        <v>0.2534</v>
       </c>
       <c r="Z6" s="22" t="n">
-        <v>0.2434</v>
+        <v>0.2504</v>
       </c>
       <c r="AA6" s="22" t="n">
-        <v>0.2193999999999999</v>
+        <v>0.2223999999999999</v>
       </c>
       <c r="AB6" s="20" t="inlineStr">
         <is>
@@ -6032,16 +6032,16 @@
         <v>1828</v>
       </c>
       <c r="AH6" s="22" t="n">
-        <v>0.419</v>
+        <v>0.4282</v>
       </c>
       <c r="AI6" s="22" t="n">
-        <v>0.3724</v>
+        <v>0.371</v>
       </c>
       <c r="AJ6" s="22" t="n">
-        <v>0.1622</v>
+        <v>0.1556</v>
       </c>
       <c r="AK6" s="22" t="n">
-        <v>0.04639999999999994</v>
+        <v>0.04519999999999999</v>
       </c>
       <c r="AL6" s="20" t="inlineStr">
         <is>
@@ -6062,16 +6062,16 @@
         <v>1605</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>0.126</v>
+        <v>0.1364</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>0.225</v>
+        <v>0.2238</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>0.3236</v>
+        <v>0.3202</v>
       </c>
       <c r="G7" s="25" t="n">
-        <v>0.3254</v>
+        <v>0.3196000000000001</v>
       </c>
       <c r="H7" s="26" t="inlineStr">
         <is>
@@ -6090,16 +6090,16 @@
         <v>1562</v>
       </c>
       <c r="N7" s="25" t="n">
-        <v>0.1086</v>
+        <v>0.1138</v>
       </c>
       <c r="O7" s="25" t="n">
-        <v>0.215</v>
+        <v>0.2168</v>
       </c>
       <c r="P7" s="25" t="n">
-        <v>0.3398</v>
+        <v>0.3476</v>
       </c>
       <c r="Q7" s="25" t="n">
-        <v>0.3366</v>
+        <v>0.3218</v>
       </c>
       <c r="R7" s="26" t="inlineStr">
         <is>
@@ -6118,16 +6118,16 @@
         <v>1729</v>
       </c>
       <c r="X7" s="25" t="n">
-        <v>0.2648</v>
+        <v>0.2592</v>
       </c>
       <c r="Y7" s="25" t="n">
-        <v>0.2606</v>
+        <v>0.2634</v>
       </c>
       <c r="Z7" s="25" t="n">
-        <v>0.2534</v>
+        <v>0.251</v>
       </c>
       <c r="AA7" s="25" t="n">
-        <v>0.2212000000000001</v>
+        <v>0.2264</v>
       </c>
       <c r="AB7" s="26" t="inlineStr">
         <is>
@@ -6146,16 +6146,16 @@
         <v>1632</v>
       </c>
       <c r="AH7" s="25" t="n">
-        <v>0.0982</v>
+        <v>0.0906</v>
       </c>
       <c r="AI7" s="25" t="n">
-        <v>0.1984</v>
+        <v>0.2076</v>
       </c>
       <c r="AJ7" s="25" t="n">
-        <v>0.4318</v>
+        <v>0.4404</v>
       </c>
       <c r="AK7" s="25" t="n">
-        <v>0.2716</v>
+        <v>0.2614</v>
       </c>
       <c r="AL7" s="26" t="inlineStr">
         <is>
@@ -6176,16 +6176,16 @@
         <v>1549</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>0.0824</v>
+        <v>0.0774</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.1512</v>
+        <v>0.1498</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.305</v>
+        <v>0.2914</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>0.4614</v>
+        <v>0.4813999999999999</v>
       </c>
       <c r="H8" s="30" t="inlineStr">
         <is>
@@ -6204,16 +6204,16 @@
         <v>1513</v>
       </c>
       <c r="N8" s="29" t="n">
-        <v>0.08359999999999999</v>
+        <v>0.07779999999999999</v>
       </c>
       <c r="O8" s="29" t="n">
-        <v>0.15</v>
+        <v>0.1524</v>
       </c>
       <c r="P8" s="29" t="n">
-        <v>0.2974</v>
+        <v>0.2846</v>
       </c>
       <c r="Q8" s="29" t="n">
-        <v>0.469</v>
+        <v>0.4852</v>
       </c>
       <c r="R8" s="30" t="inlineStr">
         <is>
@@ -6232,16 +6232,16 @@
         <v>1676</v>
       </c>
       <c r="X8" s="29" t="n">
-        <v>0.1858</v>
+        <v>0.1772</v>
       </c>
       <c r="Y8" s="29" t="n">
-        <v>0.1996</v>
+        <v>0.2086</v>
       </c>
       <c r="Z8" s="29" t="n">
-        <v>0.2748</v>
+        <v>0.2742</v>
       </c>
       <c r="AA8" s="29" t="n">
-        <v>0.3398</v>
+        <v>0.34</v>
       </c>
       <c r="AB8" s="30" t="inlineStr">
         <is>
@@ -6260,16 +6260,16 @@
         <v>1499</v>
       </c>
       <c r="AH8" s="29" t="n">
-        <v>0.0276</v>
+        <v>0.0252</v>
       </c>
       <c r="AI8" s="29" t="n">
-        <v>0.0838</v>
+        <v>0.0716</v>
       </c>
       <c r="AJ8" s="29" t="n">
-        <v>0.2538</v>
+        <v>0.2568</v>
       </c>
       <c r="AK8" s="29" t="n">
-        <v>0.6348</v>
+        <v>0.6464000000000001</v>
       </c>
       <c r="AL8" s="30" t="inlineStr">
         <is>
@@ -6474,16 +6474,16 @@
         <v>1819</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>0.494</v>
+        <v>0.4894</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.3144</v>
+        <v>0.3084</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>0.1536</v>
+        <v>0.16</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0.03800000000000001</v>
+        <v>0.04219999999999993</v>
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
@@ -6502,16 +6502,16 @@
         <v>1830</v>
       </c>
       <c r="N13" s="19" t="n">
-        <v>0.4664</v>
+        <v>0.4808</v>
       </c>
       <c r="O13" s="19" t="n">
-        <v>0.3146</v>
+        <v>0.3028</v>
       </c>
       <c r="P13" s="19" t="n">
-        <v>0.1474</v>
+        <v>0.153</v>
       </c>
       <c r="Q13" s="19" t="n">
-        <v>0.07160000000000008</v>
+        <v>0.06339999999999998</v>
       </c>
       <c r="R13" s="17" t="inlineStr">
         <is>
@@ -6530,16 +6530,16 @@
         <v>1791</v>
       </c>
       <c r="X13" s="19" t="n">
-        <v>0.4434</v>
+        <v>0.4508</v>
       </c>
       <c r="Y13" s="19" t="n">
-        <v>0.3028</v>
+        <v>0.3068</v>
       </c>
       <c r="Z13" s="19" t="n">
-        <v>0.1806</v>
+        <v>0.1716</v>
       </c>
       <c r="AA13" s="19" t="n">
-        <v>0.07319999999999996</v>
+        <v>0.0708</v>
       </c>
       <c r="AB13" s="17" t="inlineStr">
         <is>
@@ -6558,16 +6558,16 @@
         <v>1961</v>
       </c>
       <c r="AH13" s="19" t="n">
-        <v>0.7066</v>
+        <v>0.7238</v>
       </c>
       <c r="AI13" s="19" t="n">
-        <v>0.2256</v>
+        <v>0.2144</v>
       </c>
       <c r="AJ13" s="19" t="n">
-        <v>0.0572</v>
+        <v>0.0524</v>
       </c>
       <c r="AK13" s="19" t="n">
-        <v>0.0106</v>
+        <v>0.009399999999999992</v>
       </c>
       <c r="AL13" s="17" t="inlineStr">
         <is>
@@ -6588,16 +6588,16 @@
         <v>1756</v>
       </c>
       <c r="D14" s="22" t="n">
-        <v>0.3292</v>
+        <v>0.323</v>
       </c>
       <c r="E14" s="22" t="n">
-        <v>0.359</v>
+        <v>0.3582</v>
       </c>
       <c r="F14" s="22" t="n">
-        <v>0.2308</v>
+        <v>0.2436</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>0.08100000000000007</v>
+        <v>0.07520000000000002</v>
       </c>
       <c r="H14" s="20" t="inlineStr">
         <is>
@@ -6616,16 +6616,16 @@
         <v>1792</v>
       </c>
       <c r="N14" s="22" t="n">
-        <v>0.3662</v>
+        <v>0.358</v>
       </c>
       <c r="O14" s="22" t="n">
-        <v>0.339</v>
+        <v>0.347</v>
       </c>
       <c r="P14" s="22" t="n">
-        <v>0.1896</v>
+        <v>0.198</v>
       </c>
       <c r="Q14" s="22" t="n">
-        <v>0.1051999999999999</v>
+        <v>0.09700000000000003</v>
       </c>
       <c r="R14" s="20" t="inlineStr">
         <is>
@@ -6644,16 +6644,16 @@
         <v>1740</v>
       </c>
       <c r="X14" s="22" t="n">
-        <v>0.3266</v>
+        <v>0.3082</v>
       </c>
       <c r="Y14" s="22" t="n">
-        <v>0.323</v>
+        <v>0.321</v>
       </c>
       <c r="Z14" s="22" t="n">
-        <v>0.2416</v>
+        <v>0.244</v>
       </c>
       <c r="AA14" s="22" t="n">
-        <v>0.1088</v>
+        <v>0.1268</v>
       </c>
       <c r="AB14" s="20" t="inlineStr">
         <is>
@@ -6672,16 +6672,16 @@
         <v>1767</v>
       </c>
       <c r="AH14" s="22" t="n">
-        <v>0.2306</v>
+        <v>0.2142</v>
       </c>
       <c r="AI14" s="22" t="n">
-        <v>0.4768</v>
+        <v>0.4886</v>
       </c>
       <c r="AJ14" s="22" t="n">
-        <v>0.2168</v>
+        <v>0.2114</v>
       </c>
       <c r="AK14" s="22" t="n">
-        <v>0.07579999999999998</v>
+        <v>0.08580000000000007</v>
       </c>
       <c r="AL14" s="20" t="inlineStr">
         <is>
@@ -6702,16 +6702,16 @@
         <v>1647</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>0.1502</v>
+        <v>0.1618</v>
       </c>
       <c r="E15" s="25" t="n">
-        <v>0.2562</v>
+        <v>0.2606</v>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.3976</v>
+        <v>0.3932</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.196</v>
+        <v>0.1844000000000001</v>
       </c>
       <c r="H15" s="26" t="inlineStr">
         <is>
@@ -6723,23 +6723,23 @@
       </c>
       <c r="L15" s="24" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="M15" s="23" t="n">
-        <v>1610</v>
+        <v>1615</v>
       </c>
       <c r="N15" s="25" t="n">
-        <v>0.08599999999999999</v>
+        <v>0.0828</v>
       </c>
       <c r="O15" s="25" t="n">
-        <v>0.1674</v>
+        <v>0.1862</v>
       </c>
       <c r="P15" s="25" t="n">
-        <v>0.3236</v>
+        <v>0.3262</v>
       </c>
       <c r="Q15" s="25" t="n">
-        <v>0.423</v>
+        <v>0.4048</v>
       </c>
       <c r="R15" s="26" t="inlineStr">
         <is>
@@ -6758,16 +6758,16 @@
         <v>1669</v>
       </c>
       <c r="X15" s="25" t="n">
-        <v>0.1776</v>
+        <v>0.1868</v>
       </c>
       <c r="Y15" s="25" t="n">
-        <v>0.2656</v>
+        <v>0.2582</v>
       </c>
       <c r="Z15" s="25" t="n">
-        <v>0.3332</v>
+        <v>0.3368</v>
       </c>
       <c r="AA15" s="25" t="n">
-        <v>0.2236</v>
+        <v>0.2182000000000001</v>
       </c>
       <c r="AB15" s="26" t="inlineStr">
         <is>
@@ -6786,16 +6786,16 @@
         <v>1575</v>
       </c>
       <c r="AH15" s="25" t="n">
-        <v>0.041</v>
+        <v>0.0404</v>
       </c>
       <c r="AI15" s="25" t="n">
-        <v>0.179</v>
+        <v>0.1802</v>
       </c>
       <c r="AJ15" s="25" t="n">
-        <v>0.4122</v>
+        <v>0.4034</v>
       </c>
       <c r="AK15" s="25" t="n">
-        <v>0.3678</v>
+        <v>0.376</v>
       </c>
       <c r="AL15" s="26" t="inlineStr">
         <is>
@@ -6816,16 +6816,16 @@
         <v>1461</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>0.0266</v>
+        <v>0.0258</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.0704</v>
+        <v>0.0728</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>0.218</v>
+        <v>0.2032</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>0.6850000000000001</v>
+        <v>0.6981999999999999</v>
       </c>
       <c r="H16" s="30" t="inlineStr">
         <is>
@@ -6837,23 +6837,23 @@
       </c>
       <c r="L16" s="28" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="M16" s="27" t="n">
-        <v>1615</v>
+        <v>1610</v>
       </c>
       <c r="N16" s="29" t="n">
-        <v>0.0814</v>
+        <v>0.0784</v>
       </c>
       <c r="O16" s="29" t="n">
-        <v>0.179</v>
+        <v>0.164</v>
       </c>
       <c r="P16" s="29" t="n">
-        <v>0.3394</v>
+        <v>0.3228</v>
       </c>
       <c r="Q16" s="29" t="n">
-        <v>0.4002000000000001</v>
+        <v>0.4348</v>
       </c>
       <c r="R16" s="30" t="inlineStr">
         <is>
@@ -6872,16 +6872,16 @@
         <v>1532</v>
       </c>
       <c r="X16" s="29" t="n">
-        <v>0.0524</v>
+        <v>0.0542</v>
       </c>
       <c r="Y16" s="29" t="n">
-        <v>0.1086</v>
+        <v>0.114</v>
       </c>
       <c r="Z16" s="29" t="n">
-        <v>0.2446</v>
+        <v>0.2476</v>
       </c>
       <c r="AA16" s="29" t="n">
-        <v>0.5943999999999999</v>
+        <v>0.5842000000000001</v>
       </c>
       <c r="AB16" s="30" t="inlineStr">
         <is>
@@ -6900,16 +6900,16 @@
         <v>1517</v>
       </c>
       <c r="AH16" s="29" t="n">
-        <v>0.0218</v>
+        <v>0.0216</v>
       </c>
       <c r="AI16" s="29" t="n">
-        <v>0.1186</v>
+        <v>0.1168</v>
       </c>
       <c r="AJ16" s="29" t="n">
-        <v>0.3138</v>
+        <v>0.3328</v>
       </c>
       <c r="AK16" s="29" t="n">
-        <v>0.5457999999999998</v>
+        <v>0.5288</v>
       </c>
       <c r="AL16" s="30" t="inlineStr">
         <is>
@@ -7114,16 +7114,16 @@
         <v>1931</v>
       </c>
       <c r="D21" s="19" t="n">
-        <v>0.6378</v>
+        <v>0.6276</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.2402</v>
+        <v>0.2318</v>
       </c>
       <c r="F21" s="19" t="n">
-        <v>0.0868</v>
+        <v>0.1032</v>
       </c>
       <c r="G21" s="19" t="n">
-        <v>0.03519999999999997</v>
+        <v>0.03739999999999995</v>
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
@@ -7142,16 +7142,16 @@
         <v>1940</v>
       </c>
       <c r="N21" s="19" t="n">
-        <v>0.7116</v>
+        <v>0.7128</v>
       </c>
       <c r="O21" s="19" t="n">
-        <v>0.1892</v>
+        <v>0.1916</v>
       </c>
       <c r="P21" s="19" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.0726</v>
       </c>
       <c r="Q21" s="19" t="n">
-        <v>0.02379999999999999</v>
+        <v>0.02300000000000002</v>
       </c>
       <c r="R21" s="17" t="inlineStr">
         <is>
@@ -7170,16 +7170,16 @@
         <v>1832</v>
       </c>
       <c r="X21" s="19" t="n">
-        <v>0.4658</v>
+        <v>0.469</v>
       </c>
       <c r="Y21" s="19" t="n">
-        <v>0.3106</v>
+        <v>0.3074</v>
       </c>
       <c r="Z21" s="19" t="n">
-        <v>0.159</v>
+        <v>0.1518</v>
       </c>
       <c r="AA21" s="19" t="n">
-        <v>0.06460000000000002</v>
+        <v>0.07180000000000003</v>
       </c>
       <c r="AB21" s="17" t="inlineStr">
         <is>
@@ -7198,16 +7198,16 @@
         <v>1887</v>
       </c>
       <c r="AH21" s="19" t="n">
-        <v>0.5586</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="AI21" s="19" t="n">
-        <v>0.282</v>
+        <v>0.2878</v>
       </c>
       <c r="AJ21" s="19" t="n">
-        <v>0.1294</v>
+        <v>0.1226</v>
       </c>
       <c r="AK21" s="19" t="n">
-        <v>0.03000000000000005</v>
+        <v>0.03159999999999995</v>
       </c>
       <c r="AL21" s="17" t="inlineStr">
         <is>
@@ -7228,16 +7228,16 @@
         <v>1769</v>
       </c>
       <c r="D22" s="22" t="n">
-        <v>0.2142</v>
+        <v>0.2106</v>
       </c>
       <c r="E22" s="22" t="n">
-        <v>0.368</v>
+        <v>0.3704</v>
       </c>
       <c r="F22" s="22" t="n">
-        <v>0.2618</v>
+        <v>0.257</v>
       </c>
       <c r="G22" s="22" t="n">
-        <v>0.1560000000000001</v>
+        <v>0.162</v>
       </c>
       <c r="H22" s="20" t="inlineStr">
         <is>
@@ -7256,16 +7256,16 @@
         <v>1688</v>
       </c>
       <c r="N22" s="22" t="n">
-        <v>0.1274</v>
+        <v>0.1222</v>
       </c>
       <c r="O22" s="22" t="n">
-        <v>0.3336</v>
+        <v>0.3324</v>
       </c>
       <c r="P22" s="22" t="n">
-        <v>0.3094</v>
+        <v>0.305</v>
       </c>
       <c r="Q22" s="22" t="n">
-        <v>0.2296</v>
+        <v>0.2404000000000001</v>
       </c>
       <c r="R22" s="20" t="inlineStr">
         <is>
@@ -7284,16 +7284,16 @@
         <v>1794</v>
       </c>
       <c r="X22" s="22" t="n">
-        <v>0.3502</v>
+        <v>0.3492</v>
       </c>
       <c r="Y22" s="22" t="n">
-        <v>0.3456</v>
+        <v>0.3332</v>
       </c>
       <c r="Z22" s="22" t="n">
-        <v>0.2014</v>
+        <v>0.21</v>
       </c>
       <c r="AA22" s="22" t="n">
-        <v>0.1027999999999999</v>
+        <v>0.1076000000000001</v>
       </c>
       <c r="AB22" s="20" t="inlineStr">
         <is>
@@ -7312,16 +7312,16 @@
         <v>1794</v>
       </c>
       <c r="AH22" s="22" t="n">
-        <v>0.3122</v>
+        <v>0.2936</v>
       </c>
       <c r="AI22" s="22" t="n">
-        <v>0.3852</v>
+        <v>0.381</v>
       </c>
       <c r="AJ22" s="22" t="n">
-        <v>0.2294</v>
+        <v>0.2394</v>
       </c>
       <c r="AK22" s="22" t="n">
-        <v>0.07319999999999999</v>
+        <v>0.08599999999999991</v>
       </c>
       <c r="AL22" s="20" t="inlineStr">
         <is>
@@ -7342,16 +7342,16 @@
         <v>1688</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>0.1016</v>
+        <v>0.1084</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>0.2416</v>
+        <v>0.2448</v>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.3556</v>
+        <v>0.3482</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>0.3011999999999999</v>
+        <v>0.2985999999999999</v>
       </c>
       <c r="H23" s="26" t="inlineStr">
         <is>
@@ -7370,16 +7370,16 @@
         <v>1681</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>0.1128</v>
+        <v>0.1168</v>
       </c>
       <c r="O23" s="25" t="n">
-        <v>0.3098</v>
+        <v>0.3096</v>
       </c>
       <c r="P23" s="25" t="n">
-        <v>0.3294</v>
+        <v>0.3242</v>
       </c>
       <c r="Q23" s="25" t="n">
-        <v>0.2479999999999999</v>
+        <v>0.2494</v>
       </c>
       <c r="R23" s="26" t="inlineStr">
         <is>
@@ -7398,16 +7398,16 @@
         <v>1652</v>
       </c>
       <c r="X23" s="25" t="n">
-        <v>0.1086</v>
+        <v>0.1074</v>
       </c>
       <c r="Y23" s="25" t="n">
-        <v>0.1972</v>
+        <v>0.2038</v>
       </c>
       <c r="Z23" s="25" t="n">
-        <v>0.3558</v>
+        <v>0.353</v>
       </c>
       <c r="AA23" s="25" t="n">
-        <v>0.3383999999999999</v>
+        <v>0.3358000000000001</v>
       </c>
       <c r="AB23" s="26" t="inlineStr">
         <is>
@@ -7426,16 +7426,16 @@
         <v>1671</v>
       </c>
       <c r="AH23" s="25" t="n">
-        <v>0.1086</v>
+        <v>0.1264</v>
       </c>
       <c r="AI23" s="25" t="n">
-        <v>0.2556</v>
+        <v>0.2474</v>
       </c>
       <c r="AJ23" s="25" t="n">
-        <v>0.4234</v>
+        <v>0.4104</v>
       </c>
       <c r="AK23" s="25" t="n">
-        <v>0.2123999999999999</v>
+        <v>0.2157999999999999</v>
       </c>
       <c r="AL23" s="26" t="inlineStr">
         <is>
@@ -7456,16 +7456,16 @@
         <v>1613</v>
       </c>
       <c r="D24" s="29" t="n">
-        <v>0.0464</v>
+        <v>0.0534</v>
       </c>
       <c r="E24" s="29" t="n">
-        <v>0.1502</v>
+        <v>0.153</v>
       </c>
       <c r="F24" s="29" t="n">
-        <v>0.2958</v>
+        <v>0.2916</v>
       </c>
       <c r="G24" s="29" t="n">
-        <v>0.5076000000000001</v>
+        <v>0.502</v>
       </c>
       <c r="H24" s="30" t="inlineStr">
         <is>
@@ -7487,13 +7487,13 @@
         <v>0.0482</v>
       </c>
       <c r="O24" s="29" t="n">
-        <v>0.1674</v>
+        <v>0.1664</v>
       </c>
       <c r="P24" s="29" t="n">
-        <v>0.2858</v>
+        <v>0.2982</v>
       </c>
       <c r="Q24" s="29" t="n">
-        <v>0.4986</v>
+        <v>0.4872</v>
       </c>
       <c r="R24" s="30" t="inlineStr">
         <is>
@@ -7512,16 +7512,16 @@
         <v>1607</v>
       </c>
       <c r="X24" s="29" t="n">
-        <v>0.07539999999999999</v>
+        <v>0.07439999999999999</v>
       </c>
       <c r="Y24" s="29" t="n">
-        <v>0.1466</v>
+        <v>0.1556</v>
       </c>
       <c r="Z24" s="29" t="n">
-        <v>0.2838</v>
+        <v>0.2852</v>
       </c>
       <c r="AA24" s="29" t="n">
-        <v>0.4942</v>
+        <v>0.4848</v>
       </c>
       <c r="AB24" s="30" t="inlineStr">
         <is>
@@ -7540,16 +7540,16 @@
         <v>1500</v>
       </c>
       <c r="AH24" s="29" t="n">
-        <v>0.0206</v>
+        <v>0.022</v>
       </c>
       <c r="AI24" s="29" t="n">
-        <v>0.0772</v>
+        <v>0.0838</v>
       </c>
       <c r="AJ24" s="29" t="n">
-        <v>0.2178</v>
+        <v>0.2276</v>
       </c>
       <c r="AK24" s="29" t="n">
-        <v>0.6844</v>
+        <v>0.6666</v>
       </c>
       <c r="AL24" s="30" t="inlineStr">
         <is>
@@ -7718,11 +7718,11 @@
       </c>
       <c r="C5" s="33" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="D5" s="34" t="n">
-        <v>0.515</v>
+        <v>0.521</v>
       </c>
       <c r="E5" s="33" t="inlineStr">
         <is>
@@ -7730,7 +7730,7 @@
         </is>
       </c>
       <c r="F5" s="35" t="n">
-        <v>0.299</v>
+        <v>0.297</v>
       </c>
       <c r="G5" s="36" t="inlineStr">
         <is>
@@ -7755,15 +7755,15 @@
         </is>
       </c>
       <c r="D6" s="34" t="n">
-        <v>0.5379999999999999</v>
+        <v>0.54</v>
       </c>
       <c r="E6" s="33" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="F6" s="35" t="n">
-        <v>0.29</v>
+        <v>0.289</v>
       </c>
       <c r="G6" s="36" t="inlineStr">
         <is>
@@ -8048,11 +8048,11 @@
       </c>
       <c r="C15" s="33" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="D15" s="34" t="n">
-        <v>0.433</v>
+        <v>0.427</v>
       </c>
       <c r="E15" s="33" t="inlineStr">
         <is>
@@ -8060,11 +8060,11 @@
         </is>
       </c>
       <c r="F15" s="35" t="n">
-        <v>0.333</v>
+        <v>0.335</v>
       </c>
       <c r="G15" s="36" t="inlineStr">
         <is>
-          <t>→ United States</t>
+          <t>→ Turkey</t>
         </is>
       </c>
     </row>
@@ -8085,15 +8085,15 @@
         </is>
       </c>
       <c r="D16" s="34" t="n">
-        <v>0.611</v>
+        <v>0.624</v>
       </c>
       <c r="E16" s="33" t="inlineStr">
         <is>
-          <t>Algeria</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="F16" s="35" t="n">
-        <v>0.258</v>
+        <v>0.253</v>
       </c>
       <c r="G16" s="36" t="inlineStr">
         <is>
@@ -8379,11 +8379,11 @@
       </c>
       <c r="C26" s="39" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="D26" s="34" t="n">
-        <v>0.531</v>
+        <v>0.5379999999999999</v>
       </c>
       <c r="E26" s="39" t="inlineStr">
         <is>
@@ -8391,7 +8391,7 @@
         </is>
       </c>
       <c r="F26" s="35" t="n">
-        <v>0.292</v>
+        <v>0.29</v>
       </c>
       <c r="G26" s="40" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: agregar modelo ML ensemble XGBoost (Fase 4)
- Nuevo src/ml_model.py: XGBClassifier con 15 features, entrenado sobre
  37,165 partidos (1980-2026). Accuracy val 60.6%, log-loss 20.6% mejor
  que baseline. Pre-cómputo de probabilidades por pares (2,256 pares)
  para mantener velocidad de simulación (~560 torneos/s).
- src/form.py: añadir compute_form_raw() para features ML
- src/simulator.py: threading ml_model/ml_weight/form_raw/ml_cache por
  toda la cadena simulate_match → tournament → run_monte_carlo
- main.py: flags --train-ml, --ml-weight, --no-ml
- Resultados v3 (100k sims): España 23.2%, Argentina 14.7%, Francia 14.2%
- Actualizar README, CSV y Excel con resultados del ensemble

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/excel/Mundial_2026_Predicciones.xlsx
+++ b/results/excel/Mundial_2026_Predicciones.xlsx
@@ -111,7 +111,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00555555"/>
+      <color rgb="001B5E20"/>
       <sz val="10"/>
     </font>
     <font>
@@ -128,12 +128,6 @@
     <font>
       <name val="Calibri"/>
       <color rgb="00607D8B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="001B5E20"/>
       <sz val="10"/>
     </font>
     <font>
@@ -159,13 +153,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00B71C1C"/>
+      <color rgb="00555555"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00B71C1C"/>
+      <color rgb="00555555"/>
       <sz val="10"/>
     </font>
     <font>
@@ -180,7 +174,13 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <color rgb="00555555"/>
+      <color rgb="00B71C1C"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00B71C1C"/>
       <sz val="10"/>
     </font>
     <font>
@@ -534,58 +534,58 @@
     <xf numFmtId="10" fontId="18" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="10" fontId="21" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="22" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5904,16 +5904,16 @@
         <v>1762</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.4552</v>
+        <v>0.4446</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.295</v>
+        <v>0.2972</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>0.1664</v>
+        <v>0.1764</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>0.08339999999999997</v>
+        <v>0.08179999999999998</v>
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
@@ -5932,16 +5932,16 @@
         <v>1735</v>
       </c>
       <c r="N5" s="19" t="n">
-        <v>0.4888</v>
+        <v>0.502</v>
       </c>
       <c r="O5" s="19" t="n">
-        <v>0.3072</v>
+        <v>0.2958</v>
       </c>
       <c r="P5" s="19" t="n">
-        <v>0.141</v>
+        <v>0.1416</v>
       </c>
       <c r="Q5" s="19" t="n">
-        <v>0.06300000000000003</v>
+        <v>0.06059999999999999</v>
       </c>
       <c r="R5" s="17" t="inlineStr">
         <is>
@@ -5960,16 +5960,16 @@
         <v>1747</v>
       </c>
       <c r="X5" s="19" t="n">
-        <v>0.3258</v>
+        <v>0.3218</v>
       </c>
       <c r="Y5" s="19" t="n">
-        <v>0.2806</v>
+        <v>0.287</v>
       </c>
       <c r="Z5" s="19" t="n">
-        <v>0.2328</v>
+        <v>0.2314</v>
       </c>
       <c r="AA5" s="19" t="n">
-        <v>0.1608</v>
+        <v>0.1598000000000001</v>
       </c>
       <c r="AB5" s="17" t="inlineStr">
         <is>
@@ -5988,16 +5988,16 @@
         <v>1851</v>
       </c>
       <c r="AH5" s="19" t="n">
-        <v>0.5342</v>
+        <v>0.5406</v>
       </c>
       <c r="AI5" s="19" t="n">
-        <v>0.3072</v>
+        <v>0.307</v>
       </c>
       <c r="AJ5" s="19" t="n">
-        <v>0.1276</v>
+        <v>0.1198</v>
       </c>
       <c r="AK5" s="19" t="n">
-        <v>0.03100000000000003</v>
+        <v>0.03260000000000003</v>
       </c>
       <c r="AL5" s="17" t="inlineStr">
         <is>
@@ -6018,16 +6018,16 @@
         <v>1739</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>0.3562</v>
+        <v>0.363</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>0.3322</v>
+        <v>0.3352</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>0.1938</v>
+        <v>0.1968</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>0.1177999999999999</v>
+        <v>0.105</v>
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
@@ -6046,16 +6046,16 @@
         <v>1687</v>
       </c>
       <c r="N6" s="22" t="n">
-        <v>0.3488</v>
+        <v>0.3304</v>
       </c>
       <c r="O6" s="22" t="n">
-        <v>0.3536</v>
+        <v>0.3598</v>
       </c>
       <c r="P6" s="22" t="n">
-        <v>0.2006</v>
+        <v>0.2112</v>
       </c>
       <c r="Q6" s="22" t="n">
-        <v>0.09699999999999998</v>
+        <v>0.09859999999999997</v>
       </c>
       <c r="R6" s="20" t="inlineStr">
         <is>
@@ -6067,23 +6067,23 @@
       </c>
       <c r="V6" s="21" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="W6" s="20" t="n">
-        <v>1734</v>
+        <v>1706</v>
       </c>
       <c r="X6" s="22" t="n">
-        <v>0.2832</v>
+        <v>0.2858</v>
       </c>
       <c r="Y6" s="22" t="n">
-        <v>0.272</v>
+        <v>0.2808</v>
       </c>
       <c r="Z6" s="22" t="n">
-        <v>0.2454</v>
+        <v>0.246</v>
       </c>
       <c r="AA6" s="22" t="n">
-        <v>0.1994</v>
+        <v>0.1874</v>
       </c>
       <c r="AB6" s="20" t="inlineStr">
         <is>
@@ -6102,16 +6102,16 @@
         <v>1821</v>
       </c>
       <c r="AH6" s="22" t="n">
-        <v>0.3544</v>
+        <v>0.3476</v>
       </c>
       <c r="AI6" s="22" t="n">
-        <v>0.4116</v>
+        <v>0.4026</v>
       </c>
       <c r="AJ6" s="22" t="n">
-        <v>0.171</v>
+        <v>0.1864</v>
       </c>
       <c r="AK6" s="22" t="n">
-        <v>0.06299999999999992</v>
+        <v>0.06339999999999996</v>
       </c>
       <c r="AL6" s="20" t="inlineStr">
         <is>
@@ -6132,16 +6132,16 @@
         <v>1579</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>0.1086</v>
+        <v>0.1152</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>0.211</v>
+        <v>0.2044</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>0.3224</v>
+        <v>0.3346</v>
       </c>
       <c r="G7" s="25" t="n">
-        <v>0.358</v>
+        <v>0.3458</v>
       </c>
       <c r="H7" s="26" t="inlineStr">
         <is>
@@ -6160,16 +6160,16 @@
         <v>1551</v>
       </c>
       <c r="N7" s="25" t="n">
-        <v>0.0958</v>
+        <v>0.0998</v>
       </c>
       <c r="O7" s="25" t="n">
-        <v>0.1948</v>
+        <v>0.198</v>
       </c>
       <c r="P7" s="25" t="n">
-        <v>0.348</v>
+        <v>0.34</v>
       </c>
       <c r="Q7" s="25" t="n">
-        <v>0.3614000000000001</v>
+        <v>0.3621999999999999</v>
       </c>
       <c r="R7" s="26" t="inlineStr">
         <is>
@@ -6181,23 +6181,23 @@
       </c>
       <c r="V7" s="24" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="W7" s="23" t="n">
-        <v>1706</v>
+        <v>1734</v>
       </c>
       <c r="X7" s="25" t="n">
-        <v>0.272</v>
+        <v>0.2828</v>
       </c>
       <c r="Y7" s="25" t="n">
-        <v>0.2744</v>
+        <v>0.2712</v>
       </c>
       <c r="Z7" s="25" t="n">
-        <v>0.2522</v>
+        <v>0.2486</v>
       </c>
       <c r="AA7" s="25" t="n">
-        <v>0.2014</v>
+        <v>0.1974000000000001</v>
       </c>
       <c r="AB7" s="26" t="inlineStr">
         <is>
@@ -6216,16 +6216,16 @@
         <v>1611</v>
       </c>
       <c r="AH7" s="25" t="n">
-        <v>0.079</v>
+        <v>0.07920000000000001</v>
       </c>
       <c r="AI7" s="25" t="n">
-        <v>0.1758</v>
+        <v>0.1856</v>
       </c>
       <c r="AJ7" s="25" t="n">
-        <v>0.404</v>
+        <v>0.391</v>
       </c>
       <c r="AK7" s="25" t="n">
-        <v>0.3412000000000001</v>
+        <v>0.3442</v>
       </c>
       <c r="AL7" s="26" t="inlineStr">
         <is>
@@ -6246,16 +6246,16 @@
         <v>1556</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>0.08</v>
+        <v>0.0772</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.1618</v>
+        <v>0.1632</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.3174</v>
+        <v>0.2922</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>0.4408</v>
+        <v>0.4673999999999999</v>
       </c>
       <c r="H8" s="30" t="inlineStr">
         <is>
@@ -6274,16 +6274,16 @@
         <v>1475</v>
       </c>
       <c r="N8" s="29" t="n">
-        <v>0.06660000000000001</v>
+        <v>0.0678</v>
       </c>
       <c r="O8" s="29" t="n">
-        <v>0.1444</v>
+        <v>0.1464</v>
       </c>
       <c r="P8" s="29" t="n">
-        <v>0.3104</v>
+        <v>0.3072</v>
       </c>
       <c r="Q8" s="29" t="n">
-        <v>0.4786</v>
+        <v>0.4786000000000001</v>
       </c>
       <c r="R8" s="30" t="inlineStr">
         <is>
@@ -6302,16 +6302,16 @@
         <v>1637</v>
       </c>
       <c r="X8" s="29" t="n">
-        <v>0.119</v>
+        <v>0.1096</v>
       </c>
       <c r="Y8" s="29" t="n">
-        <v>0.173</v>
+        <v>0.161</v>
       </c>
       <c r="Z8" s="29" t="n">
-        <v>0.2696</v>
+        <v>0.274</v>
       </c>
       <c r="AA8" s="29" t="n">
-        <v>0.4384</v>
+        <v>0.4553999999999999</v>
       </c>
       <c r="AB8" s="30" t="inlineStr">
         <is>
@@ -6330,16 +6330,16 @@
         <v>1509</v>
       </c>
       <c r="AH8" s="29" t="n">
-        <v>0.0324</v>
+        <v>0.0326</v>
       </c>
       <c r="AI8" s="29" t="n">
-        <v>0.1054</v>
+        <v>0.1048</v>
       </c>
       <c r="AJ8" s="29" t="n">
-        <v>0.2974</v>
+        <v>0.3028</v>
       </c>
       <c r="AK8" s="29" t="n">
-        <v>0.5648000000000001</v>
+        <v>0.5598000000000001</v>
       </c>
       <c r="AL8" s="30" t="inlineStr">
         <is>
@@ -6544,16 +6544,16 @@
         <v>1806</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>0.5806</v>
+        <v>0.575</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.2548</v>
+        <v>0.2588</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>0.1232</v>
+        <v>0.1264</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0.04139999999999996</v>
+        <v>0.03980000000000006</v>
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
@@ -6572,16 +6572,16 @@
         <v>1820</v>
       </c>
       <c r="N13" s="19" t="n">
-        <v>0.4398</v>
+        <v>0.4424</v>
       </c>
       <c r="O13" s="19" t="n">
-        <v>0.3424</v>
+        <v>0.3382</v>
       </c>
       <c r="P13" s="19" t="n">
-        <v>0.157</v>
+        <v>0.1542</v>
       </c>
       <c r="Q13" s="19" t="n">
-        <v>0.06080000000000005</v>
+        <v>0.06519999999999998</v>
       </c>
       <c r="R13" s="17" t="inlineStr">
         <is>
@@ -6600,16 +6600,16 @@
         <v>1776</v>
       </c>
       <c r="X13" s="19" t="n">
-        <v>0.4516</v>
+        <v>0.4438</v>
       </c>
       <c r="Y13" s="19" t="n">
-        <v>0.2904</v>
+        <v>0.2846</v>
       </c>
       <c r="Z13" s="19" t="n">
-        <v>0.187</v>
+        <v>0.1882</v>
       </c>
       <c r="AA13" s="19" t="n">
-        <v>0.07100000000000001</v>
+        <v>0.0834</v>
       </c>
       <c r="AB13" s="17" t="inlineStr">
         <is>
@@ -6628,16 +6628,16 @@
         <v>1959</v>
       </c>
       <c r="AH13" s="19" t="n">
-        <v>0.7786</v>
+        <v>0.7678</v>
       </c>
       <c r="AI13" s="19" t="n">
-        <v>0.1714</v>
+        <v>0.187</v>
       </c>
       <c r="AJ13" s="19" t="n">
         <v>0.0392</v>
       </c>
       <c r="AK13" s="19" t="n">
-        <v>0.01080000000000005</v>
+        <v>0.005999999999999964</v>
       </c>
       <c r="AL13" s="17" t="inlineStr">
         <is>
@@ -6658,16 +6658,16 @@
         <v>1730</v>
       </c>
       <c r="D14" s="22" t="n">
-        <v>0.212</v>
+        <v>0.2056</v>
       </c>
       <c r="E14" s="22" t="n">
-        <v>0.3334</v>
+        <v>0.3456</v>
       </c>
       <c r="F14" s="22" t="n">
-        <v>0.313</v>
+        <v>0.3088</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>0.1416000000000001</v>
+        <v>0.14</v>
       </c>
       <c r="H14" s="20" t="inlineStr">
         <is>
@@ -6686,16 +6686,16 @@
         <v>1815</v>
       </c>
       <c r="N14" s="22" t="n">
-        <v>0.4358</v>
+        <v>0.4352</v>
       </c>
       <c r="O14" s="22" t="n">
-        <v>0.3562</v>
+        <v>0.3508</v>
       </c>
       <c r="P14" s="22" t="n">
-        <v>0.1498</v>
+        <v>0.1542</v>
       </c>
       <c r="Q14" s="22" t="n">
-        <v>0.05820000000000003</v>
+        <v>0.05979999999999996</v>
       </c>
       <c r="R14" s="20" t="inlineStr">
         <is>
@@ -6714,16 +6714,16 @@
         <v>1756</v>
       </c>
       <c r="X14" s="22" t="n">
-        <v>0.3182</v>
+        <v>0.3344</v>
       </c>
       <c r="Y14" s="22" t="n">
-        <v>0.3302</v>
+        <v>0.3274</v>
       </c>
       <c r="Z14" s="22" t="n">
-        <v>0.2362</v>
+        <v>0.2264</v>
       </c>
       <c r="AA14" s="22" t="n">
-        <v>0.1154</v>
+        <v>0.1118</v>
       </c>
       <c r="AB14" s="20" t="inlineStr">
         <is>
@@ -6742,16 +6742,16 @@
         <v>1745</v>
       </c>
       <c r="AH14" s="22" t="n">
-        <v>0.1622</v>
+        <v>0.1648</v>
       </c>
       <c r="AI14" s="22" t="n">
-        <v>0.4998</v>
+        <v>0.4884</v>
       </c>
       <c r="AJ14" s="22" t="n">
-        <v>0.2414</v>
+        <v>0.2494</v>
       </c>
       <c r="AK14" s="22" t="n">
-        <v>0.09659999999999996</v>
+        <v>0.09739999999999993</v>
       </c>
       <c r="AL14" s="20" t="inlineStr">
         <is>
@@ -6772,16 +6772,16 @@
         <v>1662</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>0.178</v>
+        <v>0.1882</v>
       </c>
       <c r="E15" s="25" t="n">
-        <v>0.324</v>
+        <v>0.3066</v>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.3428</v>
+        <v>0.3452</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.1552000000000001</v>
+        <v>0.16</v>
       </c>
       <c r="H15" s="26" t="inlineStr">
         <is>
@@ -6800,16 +6800,16 @@
         <v>1625</v>
       </c>
       <c r="N15" s="25" t="n">
-        <v>0.07580000000000001</v>
+        <v>0.0708</v>
       </c>
       <c r="O15" s="25" t="n">
-        <v>0.1726</v>
+        <v>0.1818</v>
       </c>
       <c r="P15" s="25" t="n">
-        <v>0.3948</v>
+        <v>0.3908</v>
       </c>
       <c r="Q15" s="25" t="n">
-        <v>0.3568000000000001</v>
+        <v>0.3566000000000001</v>
       </c>
       <c r="R15" s="26" t="inlineStr">
         <is>
@@ -6828,16 +6828,16 @@
         <v>1675</v>
       </c>
       <c r="X15" s="25" t="n">
-        <v>0.1874</v>
+        <v>0.1782</v>
       </c>
       <c r="Y15" s="25" t="n">
-        <v>0.2598</v>
+        <v>0.28</v>
       </c>
       <c r="Z15" s="25" t="n">
-        <v>0.3316</v>
+        <v>0.3392</v>
       </c>
       <c r="AA15" s="25" t="n">
-        <v>0.2212</v>
+        <v>0.2025999999999999</v>
       </c>
       <c r="AB15" s="26" t="inlineStr">
         <is>
@@ -6856,16 +6856,16 @@
         <v>1578</v>
       </c>
       <c r="AH15" s="25" t="n">
-        <v>0.0364</v>
+        <v>0.042</v>
       </c>
       <c r="AI15" s="25" t="n">
-        <v>0.193</v>
+        <v>0.1934</v>
       </c>
       <c r="AJ15" s="25" t="n">
-        <v>0.3892</v>
+        <v>0.3898</v>
       </c>
       <c r="AK15" s="25" t="n">
-        <v>0.3814</v>
+        <v>0.3748</v>
       </c>
       <c r="AL15" s="26" t="inlineStr">
         <is>
@@ -6886,16 +6886,16 @@
         <v>1491</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>0.0294</v>
+        <v>0.0312</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.0878</v>
+        <v>0.089</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>0.221</v>
+        <v>0.2196</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>0.6618000000000001</v>
+        <v>0.6602</v>
       </c>
       <c r="H16" s="30" t="inlineStr">
         <is>
@@ -6914,16 +6914,16 @@
         <v>1579</v>
       </c>
       <c r="N16" s="29" t="n">
-        <v>0.0486</v>
+        <v>0.0516</v>
       </c>
       <c r="O16" s="29" t="n">
-        <v>0.1288</v>
+        <v>0.1292</v>
       </c>
       <c r="P16" s="29" t="n">
-        <v>0.2984</v>
+        <v>0.3008</v>
       </c>
       <c r="Q16" s="29" t="n">
-        <v>0.5242</v>
+        <v>0.5184</v>
       </c>
       <c r="R16" s="30" t="inlineStr">
         <is>
@@ -6942,16 +6942,16 @@
         <v>1547</v>
       </c>
       <c r="X16" s="29" t="n">
-        <v>0.0428</v>
+        <v>0.0436</v>
       </c>
       <c r="Y16" s="29" t="n">
-        <v>0.1196</v>
+        <v>0.108</v>
       </c>
       <c r="Z16" s="29" t="n">
-        <v>0.2452</v>
+        <v>0.2462</v>
       </c>
       <c r="AA16" s="29" t="n">
-        <v>0.5924</v>
+        <v>0.6022000000000001</v>
       </c>
       <c r="AB16" s="30" t="inlineStr">
         <is>
@@ -6970,16 +6970,16 @@
         <v>1512</v>
       </c>
       <c r="AH16" s="29" t="n">
-        <v>0.0228</v>
+        <v>0.0254</v>
       </c>
       <c r="AI16" s="29" t="n">
-        <v>0.1358</v>
+        <v>0.1312</v>
       </c>
       <c r="AJ16" s="29" t="n">
-        <v>0.3302</v>
+        <v>0.3216</v>
       </c>
       <c r="AK16" s="29" t="n">
-        <v>0.5111999999999999</v>
+        <v>0.5218</v>
       </c>
       <c r="AL16" s="30" t="inlineStr">
         <is>
@@ -7184,16 +7184,16 @@
         <v>1923</v>
       </c>
       <c r="D21" s="19" t="n">
-        <v>0.588</v>
+        <v>0.609</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.2676</v>
+        <v>0.2536</v>
       </c>
       <c r="F21" s="19" t="n">
-        <v>0.1088</v>
+        <v>0.1048</v>
       </c>
       <c r="G21" s="19" t="n">
-        <v>0.03560000000000003</v>
+        <v>0.03260000000000002</v>
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
@@ -7212,16 +7212,16 @@
         <v>1925</v>
       </c>
       <c r="N21" s="19" t="n">
-        <v>0.681</v>
+        <v>0.6818</v>
       </c>
       <c r="O21" s="19" t="n">
-        <v>0.2132</v>
+        <v>0.215</v>
       </c>
       <c r="P21" s="19" t="n">
-        <v>0.081</v>
+        <v>0.0772</v>
       </c>
       <c r="Q21" s="19" t="n">
-        <v>0.02479999999999995</v>
+        <v>0.02600000000000004</v>
       </c>
       <c r="R21" s="17" t="inlineStr">
         <is>
@@ -7240,16 +7240,16 @@
         <v>1813</v>
       </c>
       <c r="X21" s="19" t="n">
-        <v>0.4714</v>
+        <v>0.4366</v>
       </c>
       <c r="Y21" s="19" t="n">
-        <v>0.2778</v>
+        <v>0.2856</v>
       </c>
       <c r="Z21" s="19" t="n">
-        <v>0.158</v>
+        <v>0.179</v>
       </c>
       <c r="AA21" s="19" t="n">
-        <v>0.09279999999999997</v>
+        <v>0.0988</v>
       </c>
       <c r="AB21" s="17" t="inlineStr">
         <is>
@@ -7268,16 +7268,16 @@
         <v>1890</v>
       </c>
       <c r="AH21" s="19" t="n">
-        <v>0.5570000000000001</v>
+        <v>0.5594</v>
       </c>
       <c r="AI21" s="19" t="n">
-        <v>0.2884</v>
+        <v>0.2938</v>
       </c>
       <c r="AJ21" s="19" t="n">
-        <v>0.1264</v>
+        <v>0.1208</v>
       </c>
       <c r="AK21" s="19" t="n">
-        <v>0.02819999999999995</v>
+        <v>0.02599999999999998</v>
       </c>
       <c r="AL21" s="17" t="inlineStr">
         <is>
@@ -7298,16 +7298,16 @@
         <v>1779</v>
       </c>
       <c r="D22" s="22" t="n">
-        <v>0.256</v>
+        <v>0.2428</v>
       </c>
       <c r="E22" s="22" t="n">
-        <v>0.3654</v>
+        <v>0.3776</v>
       </c>
       <c r="F22" s="22" t="n">
-        <v>0.2492</v>
+        <v>0.2468</v>
       </c>
       <c r="G22" s="22" t="n">
-        <v>0.1294</v>
+        <v>0.1328</v>
       </c>
       <c r="H22" s="20" t="inlineStr">
         <is>
@@ -7326,16 +7326,16 @@
         <v>1707</v>
       </c>
       <c r="N22" s="22" t="n">
-        <v>0.1536</v>
+        <v>0.1458</v>
       </c>
       <c r="O22" s="22" t="n">
-        <v>0.3404</v>
+        <v>0.3264</v>
       </c>
       <c r="P22" s="22" t="n">
-        <v>0.2988</v>
+        <v>0.317</v>
       </c>
       <c r="Q22" s="22" t="n">
-        <v>0.2072</v>
+        <v>0.2107999999999999</v>
       </c>
       <c r="R22" s="20" t="inlineStr">
         <is>
@@ -7354,16 +7354,16 @@
         <v>1781</v>
       </c>
       <c r="X22" s="22" t="n">
-        <v>0.3</v>
+        <v>0.3268</v>
       </c>
       <c r="Y22" s="22" t="n">
-        <v>0.3236</v>
+        <v>0.3194</v>
       </c>
       <c r="Z22" s="22" t="n">
-        <v>0.224</v>
+        <v>0.2062</v>
       </c>
       <c r="AA22" s="22" t="n">
-        <v>0.1524</v>
+        <v>0.1476</v>
       </c>
       <c r="AB22" s="20" t="inlineStr">
         <is>
@@ -7382,16 +7382,16 @@
         <v>1778</v>
       </c>
       <c r="AH22" s="22" t="n">
-        <v>0.298</v>
+        <v>0.2976</v>
       </c>
       <c r="AI22" s="22" t="n">
-        <v>0.3812</v>
+        <v>0.3986</v>
       </c>
       <c r="AJ22" s="22" t="n">
-        <v>0.2392</v>
+        <v>0.2274</v>
       </c>
       <c r="AK22" s="22" t="n">
-        <v>0.08159999999999998</v>
+        <v>0.07640000000000002</v>
       </c>
       <c r="AL22" s="20" t="inlineStr">
         <is>
@@ -7412,16 +7412,16 @@
         <v>1692</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>0.1062</v>
+        <v>0.1042</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>0.2262</v>
+        <v>0.2366</v>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.3658</v>
+        <v>0.3616</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>0.3018</v>
+        <v>0.2976</v>
       </c>
       <c r="H23" s="26" t="inlineStr">
         <is>
@@ -7440,16 +7440,16 @@
         <v>1663</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>0.1122</v>
+        <v>0.1138</v>
       </c>
       <c r="O23" s="25" t="n">
-        <v>0.2822</v>
+        <v>0.2858</v>
       </c>
       <c r="P23" s="25" t="n">
-        <v>0.3406</v>
+        <v>0.3272</v>
       </c>
       <c r="Q23" s="25" t="n">
-        <v>0.265</v>
+        <v>0.2732000000000001</v>
       </c>
       <c r="R23" s="26" t="inlineStr">
         <is>
@@ -7468,16 +7468,16 @@
         <v>1671</v>
       </c>
       <c r="X23" s="25" t="n">
-        <v>0.132</v>
+        <v>0.1432</v>
       </c>
       <c r="Y23" s="25" t="n">
-        <v>0.2282</v>
+        <v>0.218</v>
       </c>
       <c r="Z23" s="25" t="n">
-        <v>0.3198</v>
+        <v>0.3088</v>
       </c>
       <c r="AA23" s="25" t="n">
-        <v>0.3200000000000001</v>
+        <v>0.33</v>
       </c>
       <c r="AB23" s="26" t="inlineStr">
         <is>
@@ -7496,16 +7496,16 @@
         <v>1673</v>
       </c>
       <c r="AH23" s="25" t="n">
-        <v>0.1244</v>
+        <v>0.1236</v>
       </c>
       <c r="AI23" s="25" t="n">
-        <v>0.2574</v>
+        <v>0.237</v>
       </c>
       <c r="AJ23" s="25" t="n">
-        <v>0.412</v>
+        <v>0.43</v>
       </c>
       <c r="AK23" s="25" t="n">
-        <v>0.2062000000000001</v>
+        <v>0.2094</v>
       </c>
       <c r="AL23" s="26" t="inlineStr">
         <is>
@@ -7526,16 +7526,16 @@
         <v>1615</v>
       </c>
       <c r="D24" s="29" t="n">
-        <v>0.0498</v>
+        <v>0.044</v>
       </c>
       <c r="E24" s="29" t="n">
-        <v>0.1408</v>
+        <v>0.1322</v>
       </c>
       <c r="F24" s="29" t="n">
-        <v>0.2762</v>
+        <v>0.2868</v>
       </c>
       <c r="G24" s="29" t="n">
-        <v>0.5332</v>
+        <v>0.5369999999999999</v>
       </c>
       <c r="H24" s="30" t="inlineStr">
         <is>
@@ -7554,16 +7554,16 @@
         <v>1607</v>
       </c>
       <c r="N24" s="29" t="n">
-        <v>0.0532</v>
+        <v>0.0586</v>
       </c>
       <c r="O24" s="29" t="n">
-        <v>0.1642</v>
+        <v>0.1728</v>
       </c>
       <c r="P24" s="29" t="n">
-        <v>0.2796</v>
+        <v>0.2786</v>
       </c>
       <c r="Q24" s="29" t="n">
-        <v>0.5029999999999999</v>
+        <v>0.4899999999999999</v>
       </c>
       <c r="R24" s="30" t="inlineStr">
         <is>
@@ -7582,16 +7582,16 @@
         <v>1620</v>
       </c>
       <c r="X24" s="29" t="n">
-        <v>0.09660000000000001</v>
+        <v>0.0934</v>
       </c>
       <c r="Y24" s="29" t="n">
-        <v>0.1704</v>
+        <v>0.177</v>
       </c>
       <c r="Z24" s="29" t="n">
-        <v>0.2982</v>
+        <v>0.306</v>
       </c>
       <c r="AA24" s="29" t="n">
-        <v>0.4348</v>
+        <v>0.4236</v>
       </c>
       <c r="AB24" s="30" t="inlineStr">
         <is>
@@ -7610,16 +7610,16 @@
         <v>1508</v>
       </c>
       <c r="AH24" s="29" t="n">
-        <v>0.0206</v>
+        <v>0.0194</v>
       </c>
       <c r="AI24" s="29" t="n">
-        <v>0.073</v>
+        <v>0.0706</v>
       </c>
       <c r="AJ24" s="29" t="n">
-        <v>0.2224</v>
+        <v>0.2218</v>
       </c>
       <c r="AK24" s="29" t="n">
-        <v>0.6840000000000002</v>
+        <v>0.6882</v>
       </c>
       <c r="AL24" s="30" t="inlineStr">
         <is>
@@ -7825,15 +7825,15 @@
         </is>
       </c>
       <c r="D6" s="34" t="n">
-        <v>0.551</v>
+        <v>0.518</v>
       </c>
       <c r="E6" s="33" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F6" s="35" t="n">
-        <v>0.239</v>
+        <v>0.263</v>
       </c>
       <c r="G6" s="36" t="inlineStr">
         <is>
@@ -7858,19 +7858,19 @@
         </is>
       </c>
       <c r="D7" s="34" t="n">
-        <v>0.382</v>
+        <v>0.389</v>
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="F7" s="35" t="n">
-        <v>0.362</v>
+        <v>0.358</v>
       </c>
       <c r="G7" s="36" t="inlineStr">
         <is>
-          <t>→ Japan</t>
+          <t>→ Netherlands</t>
         </is>
       </c>
     </row>
@@ -7887,11 +7887,11 @@
       </c>
       <c r="C8" s="33" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D8" s="34" t="n">
-        <v>0.485</v>
+        <v>0.479</v>
       </c>
       <c r="E8" s="33" t="inlineStr">
         <is>
@@ -7899,11 +7899,11 @@
         </is>
       </c>
       <c r="F8" s="35" t="n">
-        <v>0.288</v>
+        <v>0.292</v>
       </c>
       <c r="G8" s="36" t="inlineStr">
         <is>
-          <t>→ Netherlands</t>
+          <t>→ Japan</t>
         </is>
       </c>
     </row>
@@ -8122,15 +8122,15 @@
         </is>
       </c>
       <c r="D15" s="34" t="n">
-        <v>0.423</v>
+        <v>0.441</v>
       </c>
       <c r="E15" s="33" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="F15" s="35" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="G15" s="36" t="inlineStr">
         <is>
@@ -8155,15 +8155,15 @@
         </is>
       </c>
       <c r="D16" s="34" t="n">
-        <v>0.5679999999999999</v>
+        <v>0.586</v>
       </c>
       <c r="E16" s="33" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="F16" s="35" t="n">
-        <v>0.227</v>
+        <v>0.213</v>
       </c>
       <c r="G16" s="36" t="inlineStr">
         <is>
@@ -8188,15 +8188,15 @@
         </is>
       </c>
       <c r="D17" s="34" t="n">
-        <v>0.498</v>
+        <v>0.5</v>
       </c>
       <c r="E17" s="33" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="F17" s="35" t="n">
-        <v>0.278</v>
+        <v>0.276</v>
       </c>
       <c r="G17" s="36" t="inlineStr">
         <is>
@@ -8221,15 +8221,15 @@
         </is>
       </c>
       <c r="D18" s="34" t="n">
-        <v>0.6940000000000001</v>
+        <v>0.696</v>
       </c>
       <c r="E18" s="33" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Uzbekistan</t>
         </is>
       </c>
       <c r="F18" s="35" t="n">
-        <v>0.134</v>
+        <v>0.132</v>
       </c>
       <c r="G18" s="36" t="inlineStr">
         <is>
@@ -8317,7 +8317,7 @@
       </c>
       <c r="C22" s="39" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="D22" s="34" t="n">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="E22" s="39" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F22" s="35" t="n">
@@ -8821,19 +8821,19 @@
         </is>
       </c>
       <c r="D3" s="55" t="n">
-        <v>0.2269</v>
+        <v>0.2285</v>
       </c>
       <c r="E3" s="55" t="n">
-        <v>0.2261</v>
+        <v>0.2316</v>
       </c>
       <c r="F3" s="56" t="inlineStr">
         <is>
-          <t>→ 0.1%</t>
+          <t>↑ 0.3%</t>
         </is>
       </c>
       <c r="G3" s="57" t="inlineStr">
         <is>
-          <t>█████████████████████████████████░░░░░░░░░░░░</t>
+          <t>██████████████████████████████████░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -8852,19 +8852,19 @@
         </is>
       </c>
       <c r="D4" s="61" t="n">
-        <v>0.1176</v>
+        <v>0.1168</v>
       </c>
       <c r="E4" s="61" t="n">
-        <v>0.1388</v>
+        <v>0.1469</v>
       </c>
       <c r="F4" s="62" t="inlineStr">
         <is>
-          <t>↑ 2.1%</t>
+          <t>↑ 3.0%</t>
         </is>
       </c>
       <c r="G4" s="63" t="inlineStr">
         <is>
-          <t>████████████████████░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>██████████████████████░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -8883,19 +8883,19 @@
         </is>
       </c>
       <c r="D5" s="67" t="n">
-        <v>0.1129</v>
+        <v>0.11</v>
       </c>
       <c r="E5" s="67" t="n">
-        <v>0.1352</v>
+        <v>0.1415</v>
       </c>
       <c r="F5" s="68" t="inlineStr">
         <is>
-          <t>↑ 2.2%</t>
+          <t>↑ 3.2%</t>
         </is>
       </c>
       <c r="G5" s="69" t="inlineStr">
         <is>
-          <t>████████████████████░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>█████████████████████░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -8914,14 +8914,14 @@
         </is>
       </c>
       <c r="D6" s="70" t="n">
-        <v>0.0863</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="E6" s="70" t="n">
-        <v>0.0805</v>
+        <v>0.0852</v>
       </c>
       <c r="F6" s="71" t="inlineStr">
         <is>
-          <t>↓ 0.6%</t>
+          <t>→ 0.0%</t>
         </is>
       </c>
       <c r="G6" s="72" t="inlineStr">
@@ -8945,14 +8945,14 @@
         </is>
       </c>
       <c r="D7" s="73" t="n">
-        <v>0.0699</v>
+        <v>0.0702</v>
       </c>
       <c r="E7" s="73" t="n">
-        <v>0.0775</v>
+        <v>0.07389999999999999</v>
       </c>
       <c r="F7" s="74" t="inlineStr">
         <is>
-          <t>↑ 0.8%</t>
+          <t>↑ 0.4%</t>
         </is>
       </c>
       <c r="G7" s="75" t="inlineStr">
@@ -8976,14 +8976,14 @@
         </is>
       </c>
       <c r="D8" s="70" t="n">
-        <v>0.031</v>
+        <v>0.0313</v>
       </c>
       <c r="E8" s="70" t="n">
-        <v>0.0406</v>
+        <v>0.0428</v>
       </c>
       <c r="F8" s="76" t="inlineStr">
         <is>
-          <t>↑ 1.0%</t>
+          <t>↑ 1.2%</t>
         </is>
       </c>
       <c r="G8" s="72" t="inlineStr">
@@ -9007,19 +9007,19 @@
         </is>
       </c>
       <c r="D9" s="73" t="n">
-        <v>0.0741</v>
+        <v>0.07480000000000001</v>
       </c>
       <c r="E9" s="73" t="n">
-        <v>0.0396</v>
+        <v>0.0428</v>
       </c>
       <c r="F9" s="77" t="inlineStr">
         <is>
-          <t>↓ 3.5%</t>
+          <t>↓ 3.2%</t>
         </is>
       </c>
       <c r="G9" s="75" t="inlineStr">
         <is>
-          <t>█████░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>██████░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -9038,19 +9038,19 @@
         </is>
       </c>
       <c r="D10" s="70" t="n">
-        <v>0.0329</v>
+        <v>0.0334</v>
       </c>
       <c r="E10" s="70" t="n">
-        <v>0.0377</v>
-      </c>
-      <c r="F10" s="76" t="inlineStr">
-        <is>
-          <t>↑ 0.5%</t>
+        <v>0.0314</v>
+      </c>
+      <c r="F10" s="71" t="inlineStr">
+        <is>
+          <t>→ 0.2%</t>
         </is>
       </c>
       <c r="G10" s="72" t="inlineStr">
         <is>
-          <t>█████░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>████░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -9069,14 +9069,14 @@
         </is>
       </c>
       <c r="D11" s="73" t="n">
-        <v>0.0203</v>
+        <v>0.0199</v>
       </c>
       <c r="E11" s="73" t="n">
-        <v>0.0288</v>
+        <v>0.0302</v>
       </c>
       <c r="F11" s="74" t="inlineStr">
         <is>
-          <t>↑ 0.9%</t>
+          <t>↑ 1.0%</t>
         </is>
       </c>
       <c r="G11" s="75" t="inlineStr">
@@ -9100,14 +9100,14 @@
         </is>
       </c>
       <c r="D12" s="70" t="n">
-        <v>0.0188</v>
+        <v>0.0193</v>
       </c>
       <c r="E12" s="70" t="n">
-        <v>0.0257</v>
+        <v>0.024</v>
       </c>
       <c r="F12" s="76" t="inlineStr">
         <is>
-          <t>↑ 0.7%</t>
+          <t>↑ 0.5%</t>
         </is>
       </c>
       <c r="G12" s="72" t="inlineStr">
@@ -9131,19 +9131,19 @@
         </is>
       </c>
       <c r="D13" s="73" t="n">
-        <v>0.023</v>
+        <v>0.0229</v>
       </c>
       <c r="E13" s="73" t="n">
-        <v>0.0215</v>
-      </c>
-      <c r="F13" s="78" t="inlineStr">
-        <is>
-          <t>→ 0.1%</t>
+        <v>0.0192</v>
+      </c>
+      <c r="F13" s="77" t="inlineStr">
+        <is>
+          <t>↓ 0.4%</t>
         </is>
       </c>
       <c r="G13" s="75" t="inlineStr">
         <is>
-          <t>███░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>██░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -9162,19 +9162,19 @@
         </is>
       </c>
       <c r="D14" s="70" t="n">
-        <v>0.0167</v>
+        <v>0.018</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>0.021</v>
-      </c>
-      <c r="F14" s="76" t="inlineStr">
-        <is>
-          <t>↑ 0.4%</t>
+        <v>0.017</v>
+      </c>
+      <c r="F14" s="71" t="inlineStr">
+        <is>
+          <t>→ 0.1%</t>
         </is>
       </c>
       <c r="G14" s="72" t="inlineStr">
         <is>
-          <t>███░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>██░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -9193,14 +9193,14 @@
         </is>
       </c>
       <c r="D15" s="73" t="n">
-        <v>0.011</v>
+        <v>0.0108</v>
       </c>
       <c r="E15" s="73" t="n">
-        <v>0.0189</v>
+        <v>0.0169</v>
       </c>
       <c r="F15" s="74" t="inlineStr">
         <is>
-          <t>↑ 0.8%</t>
+          <t>↑ 0.6%</t>
         </is>
       </c>
       <c r="G15" s="75" t="inlineStr">
@@ -9224,19 +9224,19 @@
         </is>
       </c>
       <c r="D16" s="70" t="n">
-        <v>0.0111</v>
+        <v>0.011</v>
       </c>
       <c r="E16" s="70" t="n">
-        <v>0.0128</v>
-      </c>
-      <c r="F16" s="79" t="inlineStr">
-        <is>
-          <t>→ 0.2%</t>
+        <v>0.0147</v>
+      </c>
+      <c r="F16" s="76" t="inlineStr">
+        <is>
+          <t>↑ 0.4%</t>
         </is>
       </c>
       <c r="G16" s="72" t="inlineStr">
         <is>
-          <t>█░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>██░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -9255,10 +9255,10 @@
         </is>
       </c>
       <c r="D17" s="73" t="n">
-        <v>0.0257</v>
+        <v>0.0259</v>
       </c>
       <c r="E17" s="73" t="n">
-        <v>0.0109</v>
+        <v>0.0111</v>
       </c>
       <c r="F17" s="77" t="inlineStr">
         <is>
@@ -9277,23 +9277,23 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Switzerland</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>Grupo B</t>
+          <t>Grupo A</t>
         </is>
       </c>
       <c r="D18" s="70" t="n">
-        <v>0.0101</v>
+        <v>0.018</v>
       </c>
       <c r="E18" s="70" t="n">
-        <v>0.0107</v>
-      </c>
-      <c r="F18" s="79" t="inlineStr">
-        <is>
-          <t>→ 0.1%</t>
+        <v>0.0098</v>
+      </c>
+      <c r="F18" s="78" t="inlineStr">
+        <is>
+          <t>↓ 0.8%</t>
         </is>
       </c>
       <c r="G18" s="72" t="inlineStr">
@@ -9308,23 +9308,23 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Switzerland</t>
         </is>
       </c>
       <c r="C19" s="10" t="inlineStr">
         <is>
-          <t>Grupo K</t>
+          <t>Grupo B</t>
         </is>
       </c>
       <c r="D19" s="73" t="n">
-        <v>0.0103</v>
+        <v>0.0092</v>
       </c>
       <c r="E19" s="73" t="n">
-        <v>0.0097</v>
-      </c>
-      <c r="F19" s="78" t="inlineStr">
-        <is>
-          <t>→ 0.1%</t>
+        <v>0.009000000000000001</v>
+      </c>
+      <c r="F19" s="79" t="inlineStr">
+        <is>
+          <t>→ 0.0%</t>
         </is>
       </c>
       <c r="G19" s="75" t="inlineStr">
@@ -9339,23 +9339,23 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Grupo A</t>
+          <t>Grupo K</t>
         </is>
       </c>
       <c r="D20" s="70" t="n">
-        <v>0.0181</v>
+        <v>0.0098</v>
       </c>
       <c r="E20" s="70" t="n">
-        <v>0.009300000000000001</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="F20" s="71" t="inlineStr">
         <is>
-          <t>↓ 0.9%</t>
+          <t>→ 0.1%</t>
         </is>
       </c>
       <c r="G20" s="72" t="inlineStr">
@@ -9379,19 +9379,19 @@
         </is>
       </c>
       <c r="D21" s="73" t="n">
-        <v>0.0104</v>
+        <v>0.0102</v>
       </c>
       <c r="E21" s="73" t="n">
-        <v>0.008</v>
-      </c>
-      <c r="F21" s="78" t="inlineStr">
-        <is>
-          <t>→ 0.2%</t>
+        <v>0.005600000000000001</v>
+      </c>
+      <c r="F21" s="77" t="inlineStr">
+        <is>
+          <t>↓ 0.5%</t>
         </is>
       </c>
       <c r="G21" s="75" t="inlineStr">
         <is>
-          <t>█░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -9413,16 +9413,16 @@
         <v>0.0124</v>
       </c>
       <c r="E22" s="70" t="n">
-        <v>0.0072</v>
-      </c>
-      <c r="F22" s="71" t="inlineStr">
-        <is>
-          <t>↓ 0.5%</t>
+        <v>0.0054</v>
+      </c>
+      <c r="F22" s="78" t="inlineStr">
+        <is>
+          <t>↓ 0.7%</t>
         </is>
       </c>
       <c r="G22" s="72" t="inlineStr">
         <is>
-          <t>█░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -9441,12 +9441,12 @@
         </is>
       </c>
       <c r="D23" s="73" t="n">
-        <v>0.0035</v>
+        <v>0.0039</v>
       </c>
       <c r="E23" s="73" t="n">
-        <v>0.0049</v>
-      </c>
-      <c r="F23" s="78" t="inlineStr">
+        <v>0.004500000000000001</v>
+      </c>
+      <c r="F23" s="79" t="inlineStr">
         <is>
           <t>→ 0.1%</t>
         </is>
@@ -9472,14 +9472,14 @@
         </is>
       </c>
       <c r="D24" s="70" t="n">
-        <v>0.0032</v>
+        <v>0.0028</v>
       </c>
       <c r="E24" s="70" t="n">
-        <v>0.0046</v>
-      </c>
-      <c r="F24" s="79" t="inlineStr">
-        <is>
-          <t>→ 0.1%</t>
+        <v>0.0044</v>
+      </c>
+      <c r="F24" s="71" t="inlineStr">
+        <is>
+          <t>→ 0.2%</t>
         </is>
       </c>
       <c r="G24" s="72" t="inlineStr">
@@ -9503,14 +9503,14 @@
         </is>
       </c>
       <c r="D25" s="73" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0086</v>
       </c>
       <c r="E25" s="73" t="n">
-        <v>0.0046</v>
+        <v>0.0035</v>
       </c>
       <c r="F25" s="77" t="inlineStr">
         <is>
-          <t>↓ 0.4%</t>
+          <t>↓ 0.5%</t>
         </is>
       </c>
       <c r="G25" s="75" t="inlineStr">
@@ -9537,9 +9537,9 @@
         <v>0.0063</v>
       </c>
       <c r="E26" s="70" t="n">
-        <v>0.0037</v>
-      </c>
-      <c r="F26" s="79" t="inlineStr">
+        <v>0.0033</v>
+      </c>
+      <c r="F26" s="71" t="inlineStr">
         <is>
           <t>→ 0.3%</t>
         </is>
@@ -9556,12 +9556,12 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Grupo I</t>
+          <t>Grupo B</t>
         </is>
       </c>
       <c r="D27" s="73" t="n">
@@ -9570,7 +9570,7 @@
       <c r="E27" s="73" t="n">
         <v>0.0032</v>
       </c>
-      <c r="F27" s="78" t="inlineStr">
+      <c r="F27" s="79" t="inlineStr">
         <is>
           <t>→ 0.3%</t>
         </is>
@@ -9587,23 +9587,23 @@
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Ivory Coast</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Grupo B</t>
+          <t>Grupo E</t>
         </is>
       </c>
       <c r="D28" s="70" t="n">
-        <v>0.005699999999999999</v>
+        <v>0.0049</v>
       </c>
       <c r="E28" s="70" t="n">
-        <v>0.0031</v>
-      </c>
-      <c r="F28" s="79" t="inlineStr">
-        <is>
-          <t>→ 0.3%</t>
+        <v>0.0024</v>
+      </c>
+      <c r="F28" s="71" t="inlineStr">
+        <is>
+          <t>→ 0.2%</t>
         </is>
       </c>
       <c r="G28" s="72" t="inlineStr">
@@ -9618,23 +9618,23 @@
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Ivory Coast</t>
+          <t>Norway</t>
         </is>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Grupo E</t>
+          <t>Grupo I</t>
         </is>
       </c>
       <c r="D29" s="73" t="n">
-        <v>0.004699999999999999</v>
+        <v>0.0058</v>
       </c>
       <c r="E29" s="73" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="F29" s="78" t="inlineStr">
-        <is>
-          <t>→ 0.2%</t>
+        <v>0.0024</v>
+      </c>
+      <c r="F29" s="77" t="inlineStr">
+        <is>
+          <t>↓ 0.3%</t>
         </is>
       </c>
       <c r="G29" s="75" t="inlineStr">
@@ -9658,14 +9658,14 @@
         </is>
       </c>
       <c r="D30" s="70" t="n">
-        <v>0.0021</v>
+        <v>0.002</v>
       </c>
       <c r="E30" s="70" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="F30" s="79" t="inlineStr">
-        <is>
-          <t>→ 0.1%</t>
+        <v>0.0022</v>
+      </c>
+      <c r="F30" s="71" t="inlineStr">
+        <is>
+          <t>→ 0.0%</t>
         </is>
       </c>
       <c r="G30" s="72" t="inlineStr">
@@ -9689,14 +9689,14 @@
         </is>
       </c>
       <c r="D31" s="73" t="n">
-        <v>0.0024</v>
+        <v>0.0029</v>
       </c>
       <c r="E31" s="73" t="n">
-        <v>0.0022</v>
-      </c>
-      <c r="F31" s="78" t="inlineStr">
-        <is>
-          <t>→ 0.0%</t>
+        <v>0.0016</v>
+      </c>
+      <c r="F31" s="79" t="inlineStr">
+        <is>
+          <t>→ 0.1%</t>
         </is>
       </c>
       <c r="G31" s="75" t="inlineStr">
@@ -9720,14 +9720,14 @@
         </is>
       </c>
       <c r="D32" s="70" t="n">
-        <v>0.0034</v>
+        <v>0.0036</v>
       </c>
       <c r="E32" s="70" t="n">
-        <v>0.0022</v>
-      </c>
-      <c r="F32" s="79" t="inlineStr">
-        <is>
-          <t>→ 0.1%</t>
+        <v>0.0014</v>
+      </c>
+      <c r="F32" s="71" t="inlineStr">
+        <is>
+          <t>→ 0.2%</t>
         </is>
       </c>
       <c r="G32" s="72" t="inlineStr">
@@ -9751,14 +9751,14 @@
         </is>
       </c>
       <c r="D33" s="73" t="n">
-        <v>0.0063</v>
+        <v>0.0066</v>
       </c>
       <c r="E33" s="73" t="n">
-        <v>0.0014</v>
+        <v>0.001</v>
       </c>
       <c r="F33" s="77" t="inlineStr">
         <is>
-          <t>↓ 0.5%</t>
+          <t>↓ 0.6%</t>
         </is>
       </c>
       <c r="G33" s="75" t="inlineStr">
@@ -9782,12 +9782,12 @@
         </is>
       </c>
       <c r="D34" s="70" t="n">
-        <v>0.0022</v>
+        <v>0.002</v>
       </c>
       <c r="E34" s="70" t="n">
-        <v>0.001</v>
-      </c>
-      <c r="F34" s="79" t="inlineStr">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="F34" s="71" t="inlineStr">
         <is>
           <t>→ 0.1%</t>
         </is>
@@ -9813,14 +9813,14 @@
         </is>
       </c>
       <c r="D35" s="73" t="n">
-        <v>0.0009</v>
+        <v>0.0011</v>
       </c>
       <c r="E35" s="73" t="n">
-        <v>0.0005999999999999999</v>
-      </c>
-      <c r="F35" s="78" t="inlineStr">
-        <is>
-          <t>→ 0.0%</t>
+        <v>0.0004</v>
+      </c>
+      <c r="F35" s="79" t="inlineStr">
+        <is>
+          <t>→ 0.1%</t>
         </is>
       </c>
       <c r="G35" s="75" t="inlineStr">
@@ -9844,14 +9844,14 @@
         </is>
       </c>
       <c r="D36" s="70" t="n">
-        <v>0.001</v>
+        <v>0.0009</v>
       </c>
       <c r="E36" s="70" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="F36" s="79" t="inlineStr">
-        <is>
-          <t>→ 0.1%</t>
+        <v>0.0004</v>
+      </c>
+      <c r="F36" s="71" t="inlineStr">
+        <is>
+          <t>→ 0.0%</t>
         </is>
       </c>
       <c r="G36" s="72" t="inlineStr">
@@ -9866,23 +9866,23 @@
       </c>
       <c r="B37" s="11" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Czech Republic</t>
         </is>
       </c>
       <c r="C37" s="10" t="inlineStr">
         <is>
-          <t>Grupo I</t>
+          <t>Grupo A</t>
         </is>
       </c>
       <c r="D37" s="73" t="n">
-        <v>0.0011</v>
+        <v>0.0002</v>
       </c>
       <c r="E37" s="73" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="F37" s="78" t="inlineStr">
-        <is>
-          <t>→ 0.1%</t>
+        <v>0.0003</v>
+      </c>
+      <c r="F37" s="79" t="inlineStr">
+        <is>
+          <t>→ 0.0%</t>
         </is>
       </c>
       <c r="G37" s="75" t="inlineStr">
@@ -9897,23 +9897,23 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Czech Republic</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Grupo A</t>
+          <t>Grupo I</t>
         </is>
       </c>
       <c r="D38" s="70" t="n">
-        <v>0.0002</v>
+        <v>0.0014</v>
       </c>
       <c r="E38" s="70" t="n">
-        <v>0.0004</v>
-      </c>
-      <c r="F38" s="79" t="inlineStr">
-        <is>
-          <t>→ 0.0%</t>
+        <v>0.0003</v>
+      </c>
+      <c r="F38" s="71" t="inlineStr">
+        <is>
+          <t>→ 0.1%</t>
         </is>
       </c>
       <c r="G38" s="72" t="inlineStr">
@@ -9937,14 +9937,14 @@
         </is>
       </c>
       <c r="D39" s="73" t="n">
-        <v>0.0016</v>
+        <v>0.0017</v>
       </c>
       <c r="E39" s="73" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="F39" s="78" t="inlineStr">
-        <is>
-          <t>→ 0.1%</t>
+        <v>0.0002</v>
+      </c>
+      <c r="F39" s="79" t="inlineStr">
+        <is>
+          <t>→ 0.2%</t>
         </is>
       </c>
       <c r="G39" s="75" t="inlineStr">
@@ -9971,9 +9971,9 @@
         <v>0.0005</v>
       </c>
       <c r="E40" s="70" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="F40" s="79" t="inlineStr">
+        <v>0.0002</v>
+      </c>
+      <c r="F40" s="71" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -9990,21 +9990,21 @@
       </c>
       <c r="B41" s="11" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="C41" s="10" t="inlineStr">
         <is>
-          <t>Grupo A</t>
+          <t>Grupo F</t>
         </is>
       </c>
       <c r="D41" s="73" t="n">
-        <v>0.0002</v>
+        <v>0.0001</v>
       </c>
       <c r="E41" s="73" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F41" s="78" t="inlineStr">
+      <c r="F41" s="79" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -10021,21 +10021,21 @@
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>New Zealand</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Grupo D</t>
+          <t>Grupo G</t>
         </is>
       </c>
       <c r="D42" s="70" t="n">
-        <v>0.0002</v>
+        <v>0.0003</v>
       </c>
       <c r="E42" s="70" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F42" s="79" t="inlineStr">
+      <c r="F42" s="71" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -10052,21 +10052,21 @@
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>Sweden</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>Grupo F</t>
+          <t>Grupo A</t>
         </is>
       </c>
       <c r="D43" s="73" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="E43" s="73" t="n">
         <v>0.0001</v>
       </c>
-      <c r="F43" s="78" t="inlineStr">
+      <c r="F43" s="79" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -10083,7 +10083,7 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -10095,9 +10095,9 @@
         <v>0</v>
       </c>
       <c r="E44" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="F44" s="79" t="inlineStr">
+        <v>0.0001</v>
+      </c>
+      <c r="F44" s="71" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -10114,21 +10114,21 @@
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>Grupo G</t>
+          <t>Grupo H</t>
         </is>
       </c>
       <c r="D45" s="73" t="n">
         <v>0.0002</v>
       </c>
       <c r="E45" s="73" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" s="78" t="inlineStr">
+        <v>0.0001</v>
+      </c>
+      <c r="F45" s="79" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -10145,12 +10145,12 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Cape Verde</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Grupo H</t>
+          <t>Grupo E</t>
         </is>
       </c>
       <c r="D46" s="70" t="n">
@@ -10159,7 +10159,7 @@
       <c r="E46" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="F46" s="79" t="inlineStr">
+      <c r="F46" s="71" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -10176,21 +10176,21 @@
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Cape Verde</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>Grupo E</t>
+          <t>Grupo H</t>
         </is>
       </c>
       <c r="D47" s="73" t="n">
-        <v>0</v>
+        <v>0.0001</v>
       </c>
       <c r="E47" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="F47" s="78" t="inlineStr">
+      <c r="F47" s="79" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -10207,21 +10207,21 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Haiti</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Grupo B</t>
+          <t>Grupo D</t>
         </is>
       </c>
       <c r="D48" s="70" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="E48" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="F48" s="79" t="inlineStr">
+      <c r="F48" s="71" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -10238,21 +10238,21 @@
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Grupo L</t>
+          <t>Grupo B</t>
         </is>
       </c>
       <c r="D49" s="73" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="E49" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="F49" s="78" t="inlineStr">
+      <c r="F49" s="79" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>
@@ -10269,21 +10269,21 @@
       </c>
       <c r="B50" s="5" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>Grupo H</t>
+          <t>Grupo L</t>
         </is>
       </c>
       <c r="D50" s="70" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="E50" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="F50" s="79" t="inlineStr">
+      <c r="F50" s="71" t="inlineStr">
         <is>
           <t>→ 0.0%</t>
         </is>

</xml_diff>

<commit_message>
docs: actualizar CLAUDE.md con resultados v3 y Excel regenerado
- CLAUDE.md reescrito: estado del proyecto con ML ensemble, arquitectura
  de 7 componentes, resultados v3 (top 15 con deltas ELO puro vs ensemble),
  comandos actualizados con --train-ml/--ml-weight/--no-ml
- generate_excel.py: actualizar referencias de v2 a v3
- Excel: regenerado con simulaciones v3 (España 23.2%, Argentina 14.7%)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/results/excel/Mundial_2026_Predicciones.xlsx
+++ b/results/excel/Mundial_2026_Predicciones.xlsx
@@ -5904,16 +5904,16 @@
         <v>1762</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.4446</v>
+        <v>0.443</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.2972</v>
+        <v>0.3066</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>0.1764</v>
+        <v>0.1676</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>0.08179999999999998</v>
+        <v>0.08279999999999996</v>
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
@@ -5932,16 +5932,16 @@
         <v>1735</v>
       </c>
       <c r="N5" s="19" t="n">
-        <v>0.502</v>
+        <v>0.504</v>
       </c>
       <c r="O5" s="19" t="n">
-        <v>0.2958</v>
+        <v>0.288</v>
       </c>
       <c r="P5" s="19" t="n">
-        <v>0.1416</v>
+        <v>0.1492</v>
       </c>
       <c r="Q5" s="19" t="n">
-        <v>0.06059999999999999</v>
+        <v>0.05880000000000002</v>
       </c>
       <c r="R5" s="17" t="inlineStr">
         <is>
@@ -5960,16 +5960,16 @@
         <v>1747</v>
       </c>
       <c r="X5" s="19" t="n">
-        <v>0.3218</v>
+        <v>0.3346</v>
       </c>
       <c r="Y5" s="19" t="n">
-        <v>0.287</v>
+        <v>0.277</v>
       </c>
       <c r="Z5" s="19" t="n">
-        <v>0.2314</v>
+        <v>0.2346</v>
       </c>
       <c r="AA5" s="19" t="n">
-        <v>0.1598000000000001</v>
+        <v>0.1538</v>
       </c>
       <c r="AB5" s="17" t="inlineStr">
         <is>
@@ -5991,13 +5991,13 @@
         <v>0.5406</v>
       </c>
       <c r="AI5" s="19" t="n">
-        <v>0.307</v>
+        <v>0.3104</v>
       </c>
       <c r="AJ5" s="19" t="n">
-        <v>0.1198</v>
+        <v>0.1168</v>
       </c>
       <c r="AK5" s="19" t="n">
-        <v>0.03260000000000003</v>
+        <v>0.03220000000000002</v>
       </c>
       <c r="AL5" s="17" t="inlineStr">
         <is>
@@ -6018,16 +6018,16 @@
         <v>1739</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>0.363</v>
+        <v>0.3592</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>0.3352</v>
+        <v>0.3336</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>0.1968</v>
+        <v>0.1902</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>0.105</v>
+        <v>0.117</v>
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
@@ -6046,16 +6046,16 @@
         <v>1687</v>
       </c>
       <c r="N6" s="22" t="n">
-        <v>0.3304</v>
+        <v>0.33</v>
       </c>
       <c r="O6" s="22" t="n">
-        <v>0.3598</v>
+        <v>0.3552</v>
       </c>
       <c r="P6" s="22" t="n">
-        <v>0.2112</v>
+        <v>0.2122</v>
       </c>
       <c r="Q6" s="22" t="n">
-        <v>0.09859999999999997</v>
+        <v>0.1025999999999999</v>
       </c>
       <c r="R6" s="20" t="inlineStr">
         <is>
@@ -6067,23 +6067,23 @@
       </c>
       <c r="V6" s="21" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="W6" s="20" t="n">
-        <v>1706</v>
+        <v>1734</v>
       </c>
       <c r="X6" s="22" t="n">
-        <v>0.2858</v>
+        <v>0.2862</v>
       </c>
       <c r="Y6" s="22" t="n">
-        <v>0.2808</v>
+        <v>0.269</v>
       </c>
       <c r="Z6" s="22" t="n">
-        <v>0.246</v>
+        <v>0.2456</v>
       </c>
       <c r="AA6" s="22" t="n">
-        <v>0.1874</v>
+        <v>0.1992</v>
       </c>
       <c r="AB6" s="20" t="inlineStr">
         <is>
@@ -6102,16 +6102,16 @@
         <v>1821</v>
       </c>
       <c r="AH6" s="22" t="n">
-        <v>0.3476</v>
+        <v>0.3534</v>
       </c>
       <c r="AI6" s="22" t="n">
-        <v>0.4026</v>
+        <v>0.404</v>
       </c>
       <c r="AJ6" s="22" t="n">
-        <v>0.1864</v>
+        <v>0.1758</v>
       </c>
       <c r="AK6" s="22" t="n">
-        <v>0.06339999999999996</v>
+        <v>0.06680000000000003</v>
       </c>
       <c r="AL6" s="20" t="inlineStr">
         <is>
@@ -6132,16 +6132,16 @@
         <v>1579</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>0.1152</v>
+        <v>0.114</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>0.2044</v>
+        <v>0.202</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>0.3346</v>
+        <v>0.3382</v>
       </c>
       <c r="G7" s="25" t="n">
-        <v>0.3458</v>
+        <v>0.3457999999999999</v>
       </c>
       <c r="H7" s="26" t="inlineStr">
         <is>
@@ -6160,16 +6160,16 @@
         <v>1551</v>
       </c>
       <c r="N7" s="25" t="n">
-        <v>0.0998</v>
+        <v>0.1026</v>
       </c>
       <c r="O7" s="25" t="n">
-        <v>0.198</v>
+        <v>0.205</v>
       </c>
       <c r="P7" s="25" t="n">
-        <v>0.34</v>
+        <v>0.3502</v>
       </c>
       <c r="Q7" s="25" t="n">
-        <v>0.3621999999999999</v>
+        <v>0.3422</v>
       </c>
       <c r="R7" s="26" t="inlineStr">
         <is>
@@ -6181,23 +6181,23 @@
       </c>
       <c r="V7" s="24" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="W7" s="23" t="n">
-        <v>1734</v>
+        <v>1706</v>
       </c>
       <c r="X7" s="25" t="n">
-        <v>0.2828</v>
+        <v>0.2698</v>
       </c>
       <c r="Y7" s="25" t="n">
-        <v>0.2712</v>
+        <v>0.2806</v>
       </c>
       <c r="Z7" s="25" t="n">
-        <v>0.2486</v>
+        <v>0.259</v>
       </c>
       <c r="AA7" s="25" t="n">
-        <v>0.1974000000000001</v>
+        <v>0.1905999999999999</v>
       </c>
       <c r="AB7" s="26" t="inlineStr">
         <is>
@@ -6216,16 +6216,16 @@
         <v>1611</v>
       </c>
       <c r="AH7" s="25" t="n">
-        <v>0.07920000000000001</v>
+        <v>0.07340000000000001</v>
       </c>
       <c r="AI7" s="25" t="n">
-        <v>0.1856</v>
+        <v>0.1814</v>
       </c>
       <c r="AJ7" s="25" t="n">
-        <v>0.391</v>
+        <v>0.4084</v>
       </c>
       <c r="AK7" s="25" t="n">
-        <v>0.3442</v>
+        <v>0.3368</v>
       </c>
       <c r="AL7" s="26" t="inlineStr">
         <is>
@@ -6246,16 +6246,16 @@
         <v>1556</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>0.0772</v>
+        <v>0.0838</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.1632</v>
+        <v>0.1578</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.2922</v>
+        <v>0.304</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>0.4673999999999999</v>
+        <v>0.4544</v>
       </c>
       <c r="H8" s="30" t="inlineStr">
         <is>
@@ -6274,16 +6274,16 @@
         <v>1475</v>
       </c>
       <c r="N8" s="29" t="n">
-        <v>0.0678</v>
+        <v>0.0634</v>
       </c>
       <c r="O8" s="29" t="n">
-        <v>0.1464</v>
+        <v>0.1518</v>
       </c>
       <c r="P8" s="29" t="n">
-        <v>0.3072</v>
+        <v>0.2884</v>
       </c>
       <c r="Q8" s="29" t="n">
-        <v>0.4786000000000001</v>
+        <v>0.4964</v>
       </c>
       <c r="R8" s="30" t="inlineStr">
         <is>
@@ -6302,16 +6302,16 @@
         <v>1637</v>
       </c>
       <c r="X8" s="29" t="n">
-        <v>0.1096</v>
+        <v>0.1094</v>
       </c>
       <c r="Y8" s="29" t="n">
-        <v>0.161</v>
+        <v>0.1734</v>
       </c>
       <c r="Z8" s="29" t="n">
-        <v>0.274</v>
+        <v>0.2608</v>
       </c>
       <c r="AA8" s="29" t="n">
-        <v>0.4553999999999999</v>
+        <v>0.4564000000000001</v>
       </c>
       <c r="AB8" s="30" t="inlineStr">
         <is>
@@ -6333,13 +6333,13 @@
         <v>0.0326</v>
       </c>
       <c r="AI8" s="29" t="n">
-        <v>0.1048</v>
+        <v>0.1042</v>
       </c>
       <c r="AJ8" s="29" t="n">
-        <v>0.3028</v>
+        <v>0.299</v>
       </c>
       <c r="AK8" s="29" t="n">
-        <v>0.5598000000000001</v>
+        <v>0.5642</v>
       </c>
       <c r="AL8" s="30" t="inlineStr">
         <is>
@@ -6544,16 +6544,16 @@
         <v>1806</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>0.575</v>
+        <v>0.5738</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.2588</v>
+        <v>0.2678</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>0.1264</v>
+        <v>0.1228</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0.03980000000000006</v>
+        <v>0.03560000000000003</v>
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
@@ -6565,23 +6565,23 @@
       </c>
       <c r="L13" s="18" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="M13" s="17" t="n">
-        <v>1820</v>
+        <v>1815</v>
       </c>
       <c r="N13" s="19" t="n">
-        <v>0.4424</v>
+        <v>0.4496</v>
       </c>
       <c r="O13" s="19" t="n">
-        <v>0.3382</v>
+        <v>0.3458</v>
       </c>
       <c r="P13" s="19" t="n">
-        <v>0.1542</v>
+        <v>0.1478</v>
       </c>
       <c r="Q13" s="19" t="n">
-        <v>0.06519999999999998</v>
+        <v>0.05680000000000002</v>
       </c>
       <c r="R13" s="17" t="inlineStr">
         <is>
@@ -6600,16 +6600,16 @@
         <v>1776</v>
       </c>
       <c r="X13" s="19" t="n">
-        <v>0.4438</v>
+        <v>0.445</v>
       </c>
       <c r="Y13" s="19" t="n">
-        <v>0.2846</v>
+        <v>0.2894</v>
       </c>
       <c r="Z13" s="19" t="n">
-        <v>0.1882</v>
+        <v>0.188</v>
       </c>
       <c r="AA13" s="19" t="n">
-        <v>0.0834</v>
+        <v>0.07759999999999995</v>
       </c>
       <c r="AB13" s="17" t="inlineStr">
         <is>
@@ -6628,16 +6628,16 @@
         <v>1959</v>
       </c>
       <c r="AH13" s="19" t="n">
-        <v>0.7678</v>
+        <v>0.781</v>
       </c>
       <c r="AI13" s="19" t="n">
-        <v>0.187</v>
+        <v>0.176</v>
       </c>
       <c r="AJ13" s="19" t="n">
-        <v>0.0392</v>
+        <v>0.0358</v>
       </c>
       <c r="AK13" s="19" t="n">
-        <v>0.005999999999999964</v>
+        <v>0.007199999999999984</v>
       </c>
       <c r="AL13" s="17" t="inlineStr">
         <is>
@@ -6658,16 +6658,16 @@
         <v>1730</v>
       </c>
       <c r="D14" s="22" t="n">
-        <v>0.2056</v>
+        <v>0.2084</v>
       </c>
       <c r="E14" s="22" t="n">
-        <v>0.3456</v>
+        <v>0.339</v>
       </c>
       <c r="F14" s="22" t="n">
-        <v>0.3088</v>
+        <v>0.313</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>0.14</v>
+        <v>0.1395999999999999</v>
       </c>
       <c r="H14" s="20" t="inlineStr">
         <is>
@@ -6679,23 +6679,23 @@
       </c>
       <c r="L14" s="21" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="M14" s="20" t="n">
-        <v>1815</v>
+        <v>1820</v>
       </c>
       <c r="N14" s="22" t="n">
-        <v>0.4352</v>
+        <v>0.4262</v>
       </c>
       <c r="O14" s="22" t="n">
-        <v>0.3508</v>
+        <v>0.3486</v>
       </c>
       <c r="P14" s="22" t="n">
-        <v>0.1542</v>
+        <v>0.1592</v>
       </c>
       <c r="Q14" s="22" t="n">
-        <v>0.05979999999999996</v>
+        <v>0.06599999999999995</v>
       </c>
       <c r="R14" s="20" t="inlineStr">
         <is>
@@ -6714,16 +6714,16 @@
         <v>1756</v>
       </c>
       <c r="X14" s="22" t="n">
-        <v>0.3344</v>
+        <v>0.3214</v>
       </c>
       <c r="Y14" s="22" t="n">
-        <v>0.3274</v>
+        <v>0.323</v>
       </c>
       <c r="Z14" s="22" t="n">
-        <v>0.2264</v>
+        <v>0.2382</v>
       </c>
       <c r="AA14" s="22" t="n">
-        <v>0.1118</v>
+        <v>0.1174</v>
       </c>
       <c r="AB14" s="20" t="inlineStr">
         <is>
@@ -6742,16 +6742,16 @@
         <v>1745</v>
       </c>
       <c r="AH14" s="22" t="n">
-        <v>0.1648</v>
+        <v>0.1584</v>
       </c>
       <c r="AI14" s="22" t="n">
-        <v>0.4884</v>
+        <v>0.499</v>
       </c>
       <c r="AJ14" s="22" t="n">
-        <v>0.2494</v>
+        <v>0.2406</v>
       </c>
       <c r="AK14" s="22" t="n">
-        <v>0.09739999999999993</v>
+        <v>0.102</v>
       </c>
       <c r="AL14" s="20" t="inlineStr">
         <is>
@@ -6772,16 +6772,16 @@
         <v>1662</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>0.1882</v>
+        <v>0.1914</v>
       </c>
       <c r="E15" s="25" t="n">
-        <v>0.3066</v>
+        <v>0.3006</v>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.3452</v>
+        <v>0.3406</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.16</v>
+        <v>0.1674</v>
       </c>
       <c r="H15" s="26" t="inlineStr">
         <is>
@@ -6800,16 +6800,16 @@
         <v>1625</v>
       </c>
       <c r="N15" s="25" t="n">
-        <v>0.0708</v>
+        <v>0.074</v>
       </c>
       <c r="O15" s="25" t="n">
-        <v>0.1818</v>
+        <v>0.1778</v>
       </c>
       <c r="P15" s="25" t="n">
-        <v>0.3908</v>
+        <v>0.4084</v>
       </c>
       <c r="Q15" s="25" t="n">
-        <v>0.3566000000000001</v>
+        <v>0.3398</v>
       </c>
       <c r="R15" s="26" t="inlineStr">
         <is>
@@ -6828,16 +6828,16 @@
         <v>1675</v>
       </c>
       <c r="X15" s="25" t="n">
-        <v>0.1782</v>
+        <v>0.1806</v>
       </c>
       <c r="Y15" s="25" t="n">
-        <v>0.28</v>
+        <v>0.2822</v>
       </c>
       <c r="Z15" s="25" t="n">
-        <v>0.3392</v>
+        <v>0.3304</v>
       </c>
       <c r="AA15" s="25" t="n">
-        <v>0.2025999999999999</v>
+        <v>0.2068</v>
       </c>
       <c r="AB15" s="26" t="inlineStr">
         <is>
@@ -6856,16 +6856,16 @@
         <v>1578</v>
       </c>
       <c r="AH15" s="25" t="n">
-        <v>0.042</v>
+        <v>0.0412</v>
       </c>
       <c r="AI15" s="25" t="n">
-        <v>0.1934</v>
+        <v>0.197</v>
       </c>
       <c r="AJ15" s="25" t="n">
-        <v>0.3898</v>
+        <v>0.3856</v>
       </c>
       <c r="AK15" s="25" t="n">
-        <v>0.3748</v>
+        <v>0.3762</v>
       </c>
       <c r="AL15" s="26" t="inlineStr">
         <is>
@@ -6886,16 +6886,16 @@
         <v>1491</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>0.0312</v>
+        <v>0.0264</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.089</v>
+        <v>0.0926</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>0.2196</v>
+        <v>0.2236</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>0.6602</v>
+        <v>0.6574</v>
       </c>
       <c r="H16" s="30" t="inlineStr">
         <is>
@@ -6914,16 +6914,16 @@
         <v>1579</v>
       </c>
       <c r="N16" s="29" t="n">
-        <v>0.0516</v>
+        <v>0.0502</v>
       </c>
       <c r="O16" s="29" t="n">
-        <v>0.1292</v>
+        <v>0.1278</v>
       </c>
       <c r="P16" s="29" t="n">
-        <v>0.3008</v>
+        <v>0.2846</v>
       </c>
       <c r="Q16" s="29" t="n">
-        <v>0.5184</v>
+        <v>0.5373999999999999</v>
       </c>
       <c r="R16" s="30" t="inlineStr">
         <is>
@@ -6942,16 +6942,16 @@
         <v>1547</v>
       </c>
       <c r="X16" s="29" t="n">
-        <v>0.0436</v>
+        <v>0.053</v>
       </c>
       <c r="Y16" s="29" t="n">
-        <v>0.108</v>
+        <v>0.1054</v>
       </c>
       <c r="Z16" s="29" t="n">
-        <v>0.2462</v>
+        <v>0.2434</v>
       </c>
       <c r="AA16" s="29" t="n">
-        <v>0.6022000000000001</v>
+        <v>0.5981999999999998</v>
       </c>
       <c r="AB16" s="30" t="inlineStr">
         <is>
@@ -6970,16 +6970,16 @@
         <v>1512</v>
       </c>
       <c r="AH16" s="29" t="n">
-        <v>0.0254</v>
+        <v>0.0194</v>
       </c>
       <c r="AI16" s="29" t="n">
-        <v>0.1312</v>
+        <v>0.128</v>
       </c>
       <c r="AJ16" s="29" t="n">
-        <v>0.3216</v>
+        <v>0.338</v>
       </c>
       <c r="AK16" s="29" t="n">
-        <v>0.5218</v>
+        <v>0.5145999999999999</v>
       </c>
       <c r="AL16" s="30" t="inlineStr">
         <is>
@@ -7184,16 +7184,16 @@
         <v>1923</v>
       </c>
       <c r="D21" s="19" t="n">
-        <v>0.609</v>
+        <v>0.6088</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.2536</v>
+        <v>0.248</v>
       </c>
       <c r="F21" s="19" t="n">
-        <v>0.1048</v>
+        <v>0.1076</v>
       </c>
       <c r="G21" s="19" t="n">
-        <v>0.03260000000000002</v>
+        <v>0.03559999999999999</v>
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
@@ -7212,16 +7212,16 @@
         <v>1925</v>
       </c>
       <c r="N21" s="19" t="n">
-        <v>0.6818</v>
+        <v>0.6844</v>
       </c>
       <c r="O21" s="19" t="n">
-        <v>0.215</v>
+        <v>0.214</v>
       </c>
       <c r="P21" s="19" t="n">
-        <v>0.0772</v>
+        <v>0.0752</v>
       </c>
       <c r="Q21" s="19" t="n">
-        <v>0.02600000000000004</v>
+        <v>0.02639999999999999</v>
       </c>
       <c r="R21" s="17" t="inlineStr">
         <is>
@@ -7240,16 +7240,16 @@
         <v>1813</v>
       </c>
       <c r="X21" s="19" t="n">
-        <v>0.4366</v>
+        <v>0.4466</v>
       </c>
       <c r="Y21" s="19" t="n">
-        <v>0.2856</v>
+        <v>0.289</v>
       </c>
       <c r="Z21" s="19" t="n">
-        <v>0.179</v>
+        <v>0.168</v>
       </c>
       <c r="AA21" s="19" t="n">
-        <v>0.0988</v>
+        <v>0.09640000000000001</v>
       </c>
       <c r="AB21" s="17" t="inlineStr">
         <is>
@@ -7268,16 +7268,16 @@
         <v>1890</v>
       </c>
       <c r="AH21" s="19" t="n">
-        <v>0.5594</v>
+        <v>0.5648</v>
       </c>
       <c r="AI21" s="19" t="n">
-        <v>0.2938</v>
+        <v>0.2808</v>
       </c>
       <c r="AJ21" s="19" t="n">
-        <v>0.1208</v>
+        <v>0.1272</v>
       </c>
       <c r="AK21" s="19" t="n">
-        <v>0.02599999999999998</v>
+        <v>0.02720000000000003</v>
       </c>
       <c r="AL21" s="17" t="inlineStr">
         <is>
@@ -7298,16 +7298,16 @@
         <v>1779</v>
       </c>
       <c r="D22" s="22" t="n">
-        <v>0.2428</v>
+        <v>0.2364</v>
       </c>
       <c r="E22" s="22" t="n">
-        <v>0.3776</v>
+        <v>0.3638</v>
       </c>
       <c r="F22" s="22" t="n">
-        <v>0.2468</v>
+        <v>0.264</v>
       </c>
       <c r="G22" s="22" t="n">
-        <v>0.1328</v>
+        <v>0.1358</v>
       </c>
       <c r="H22" s="20" t="inlineStr">
         <is>
@@ -7326,16 +7326,16 @@
         <v>1707</v>
       </c>
       <c r="N22" s="22" t="n">
-        <v>0.1458</v>
+        <v>0.1496</v>
       </c>
       <c r="O22" s="22" t="n">
-        <v>0.3264</v>
+        <v>0.3412</v>
       </c>
       <c r="P22" s="22" t="n">
-        <v>0.317</v>
+        <v>0.304</v>
       </c>
       <c r="Q22" s="22" t="n">
-        <v>0.2107999999999999</v>
+        <v>0.2052000000000001</v>
       </c>
       <c r="R22" s="20" t="inlineStr">
         <is>
@@ -7354,16 +7354,16 @@
         <v>1781</v>
       </c>
       <c r="X22" s="22" t="n">
-        <v>0.3268</v>
+        <v>0.3138</v>
       </c>
       <c r="Y22" s="22" t="n">
-        <v>0.3194</v>
+        <v>0.3082</v>
       </c>
       <c r="Z22" s="22" t="n">
-        <v>0.2062</v>
+        <v>0.233</v>
       </c>
       <c r="AA22" s="22" t="n">
-        <v>0.1476</v>
+        <v>0.1449999999999999</v>
       </c>
       <c r="AB22" s="20" t="inlineStr">
         <is>
@@ -7382,16 +7382,16 @@
         <v>1778</v>
       </c>
       <c r="AH22" s="22" t="n">
-        <v>0.2976</v>
+        <v>0.2998</v>
       </c>
       <c r="AI22" s="22" t="n">
-        <v>0.3986</v>
+        <v>0.3852</v>
       </c>
       <c r="AJ22" s="22" t="n">
-        <v>0.2274</v>
+        <v>0.2352</v>
       </c>
       <c r="AK22" s="22" t="n">
-        <v>0.07640000000000002</v>
+        <v>0.07979999999999995</v>
       </c>
       <c r="AL22" s="20" t="inlineStr">
         <is>
@@ -7412,16 +7412,16 @@
         <v>1692</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>0.1042</v>
+        <v>0.1032</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>0.2366</v>
+        <v>0.2478</v>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.3616</v>
+        <v>0.3522</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>0.2976</v>
+        <v>0.2968</v>
       </c>
       <c r="H23" s="26" t="inlineStr">
         <is>
@@ -7440,16 +7440,16 @@
         <v>1663</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>0.1138</v>
+        <v>0.1104</v>
       </c>
       <c r="O23" s="25" t="n">
-        <v>0.2858</v>
+        <v>0.281</v>
       </c>
       <c r="P23" s="25" t="n">
-        <v>0.3272</v>
+        <v>0.337</v>
       </c>
       <c r="Q23" s="25" t="n">
-        <v>0.2732000000000001</v>
+        <v>0.2715999999999999</v>
       </c>
       <c r="R23" s="26" t="inlineStr">
         <is>
@@ -7468,16 +7468,16 @@
         <v>1671</v>
       </c>
       <c r="X23" s="25" t="n">
-        <v>0.1432</v>
+        <v>0.1396</v>
       </c>
       <c r="Y23" s="25" t="n">
-        <v>0.218</v>
+        <v>0.2202</v>
       </c>
       <c r="Z23" s="25" t="n">
-        <v>0.3088</v>
+        <v>0.3144</v>
       </c>
       <c r="AA23" s="25" t="n">
-        <v>0.33</v>
+        <v>0.3258000000000001</v>
       </c>
       <c r="AB23" s="26" t="inlineStr">
         <is>
@@ -7496,16 +7496,16 @@
         <v>1673</v>
       </c>
       <c r="AH23" s="25" t="n">
-        <v>0.1236</v>
+        <v>0.1148</v>
       </c>
       <c r="AI23" s="25" t="n">
-        <v>0.237</v>
+        <v>0.2612</v>
       </c>
       <c r="AJ23" s="25" t="n">
-        <v>0.43</v>
+        <v>0.4204</v>
       </c>
       <c r="AK23" s="25" t="n">
-        <v>0.2094</v>
+        <v>0.2036</v>
       </c>
       <c r="AL23" s="26" t="inlineStr">
         <is>
@@ -7526,16 +7526,16 @@
         <v>1615</v>
       </c>
       <c r="D24" s="29" t="n">
-        <v>0.044</v>
+        <v>0.0516</v>
       </c>
       <c r="E24" s="29" t="n">
-        <v>0.1322</v>
+        <v>0.1404</v>
       </c>
       <c r="F24" s="29" t="n">
-        <v>0.2868</v>
+        <v>0.2762</v>
       </c>
       <c r="G24" s="29" t="n">
-        <v>0.5369999999999999</v>
+        <v>0.5318000000000001</v>
       </c>
       <c r="H24" s="30" t="inlineStr">
         <is>
@@ -7554,16 +7554,16 @@
         <v>1607</v>
       </c>
       <c r="N24" s="29" t="n">
-        <v>0.0586</v>
+        <v>0.0556</v>
       </c>
       <c r="O24" s="29" t="n">
-        <v>0.1728</v>
+        <v>0.1638</v>
       </c>
       <c r="P24" s="29" t="n">
-        <v>0.2786</v>
+        <v>0.2838</v>
       </c>
       <c r="Q24" s="29" t="n">
-        <v>0.4899999999999999</v>
+        <v>0.4968</v>
       </c>
       <c r="R24" s="30" t="inlineStr">
         <is>
@@ -7582,16 +7582,16 @@
         <v>1620</v>
       </c>
       <c r="X24" s="29" t="n">
-        <v>0.0934</v>
+        <v>0.1</v>
       </c>
       <c r="Y24" s="29" t="n">
-        <v>0.177</v>
+        <v>0.1826</v>
       </c>
       <c r="Z24" s="29" t="n">
-        <v>0.306</v>
+        <v>0.2846</v>
       </c>
       <c r="AA24" s="29" t="n">
-        <v>0.4236</v>
+        <v>0.4328</v>
       </c>
       <c r="AB24" s="30" t="inlineStr">
         <is>
@@ -7610,16 +7610,16 @@
         <v>1508</v>
       </c>
       <c r="AH24" s="29" t="n">
-        <v>0.0194</v>
+        <v>0.0206</v>
       </c>
       <c r="AI24" s="29" t="n">
-        <v>0.0706</v>
+        <v>0.0728</v>
       </c>
       <c r="AJ24" s="29" t="n">
-        <v>0.2218</v>
+        <v>0.2172</v>
       </c>
       <c r="AK24" s="29" t="n">
-        <v>0.6882</v>
+        <v>0.6894</v>
       </c>
       <c r="AL24" s="30" t="inlineStr">
         <is>
@@ -7825,15 +7825,15 @@
         </is>
       </c>
       <c r="D6" s="34" t="n">
-        <v>0.518</v>
+        <v>0.551</v>
       </c>
       <c r="E6" s="33" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="F6" s="35" t="n">
-        <v>0.263</v>
+        <v>0.239</v>
       </c>
       <c r="G6" s="36" t="inlineStr">
         <is>
@@ -7858,19 +7858,19 @@
         </is>
       </c>
       <c r="D7" s="34" t="n">
-        <v>0.389</v>
+        <v>0.382</v>
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="F7" s="35" t="n">
-        <v>0.358</v>
+        <v>0.362</v>
       </c>
       <c r="G7" s="36" t="inlineStr">
         <is>
-          <t>→ Netherlands</t>
+          <t>→ Japan</t>
         </is>
       </c>
     </row>
@@ -8089,15 +8089,15 @@
         </is>
       </c>
       <c r="D14" s="34" t="n">
-        <v>0.508</v>
+        <v>0.468</v>
       </c>
       <c r="E14" s="33" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="F14" s="35" t="n">
-        <v>0.271</v>
+        <v>0.301</v>
       </c>
       <c r="G14" s="36" t="inlineStr">
         <is>
@@ -8317,23 +8317,23 @@
       </c>
       <c r="C22" s="39" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D22" s="34" t="n">
-        <v>0.377</v>
+        <v>0.371</v>
       </c>
       <c r="E22" s="39" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="F22" s="35" t="n">
-        <v>0.366</v>
+      <c r="F22" s="34" t="n">
+        <v>0.371</v>
       </c>
       <c r="G22" s="40" t="inlineStr">
         <is>
-          <t>→ Netherlands</t>
+          <t>→ Japan</t>
         </is>
       </c>
     </row>
@@ -8549,11 +8549,11 @@
       </c>
       <c r="C30" s="43" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D30" s="34" t="n">
-        <v>0.544</v>
+        <v>0.55</v>
       </c>
       <c r="E30" s="43" t="inlineStr">
         <is>
@@ -8561,7 +8561,7 @@
         </is>
       </c>
       <c r="F30" s="35" t="n">
-        <v>0.244</v>
+        <v>0.24</v>
       </c>
       <c r="G30" s="44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
fix(bracket): corregir swap de probabilidades en proyecciones y generar dashboard interactivo
</commit_message>
<xml_diff>
--- a/results/excel/Mundial_2026_Predicciones.xlsx
+++ b/results/excel/Mundial_2026_Predicciones.xlsx
@@ -576,13 +576,13 @@
     <xf numFmtId="0" fontId="25" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5904,16 +5904,16 @@
         <v>1762</v>
       </c>
       <c r="D5" s="19" t="n">
-        <v>0.443</v>
+        <v>0.4424</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>0.3066</v>
+        <v>0.3118</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>0.1676</v>
+        <v>0.1604</v>
       </c>
       <c r="G5" s="19" t="n">
-        <v>0.08279999999999996</v>
+        <v>0.08539999999999998</v>
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
@@ -5932,16 +5932,16 @@
         <v>1735</v>
       </c>
       <c r="N5" s="19" t="n">
-        <v>0.504</v>
+        <v>0.493</v>
       </c>
       <c r="O5" s="19" t="n">
-        <v>0.288</v>
+        <v>0.2984</v>
       </c>
       <c r="P5" s="19" t="n">
-        <v>0.1492</v>
+        <v>0.1396</v>
       </c>
       <c r="Q5" s="19" t="n">
-        <v>0.05880000000000002</v>
+        <v>0.06900000000000001</v>
       </c>
       <c r="R5" s="17" t="inlineStr">
         <is>
@@ -5960,16 +5960,16 @@
         <v>1747</v>
       </c>
       <c r="X5" s="19" t="n">
-        <v>0.3346</v>
+        <v>0.3432</v>
       </c>
       <c r="Y5" s="19" t="n">
-        <v>0.277</v>
+        <v>0.2562</v>
       </c>
       <c r="Z5" s="19" t="n">
-        <v>0.2346</v>
+        <v>0.2434</v>
       </c>
       <c r="AA5" s="19" t="n">
-        <v>0.1538</v>
+        <v>0.1572000000000001</v>
       </c>
       <c r="AB5" s="17" t="inlineStr">
         <is>
@@ -5988,16 +5988,16 @@
         <v>1851</v>
       </c>
       <c r="AH5" s="19" t="n">
-        <v>0.5406</v>
+        <v>0.527</v>
       </c>
       <c r="AI5" s="19" t="n">
-        <v>0.3104</v>
+        <v>0.3218</v>
       </c>
       <c r="AJ5" s="19" t="n">
-        <v>0.1168</v>
+        <v>0.1202</v>
       </c>
       <c r="AK5" s="19" t="n">
-        <v>0.03220000000000002</v>
+        <v>0.031</v>
       </c>
       <c r="AL5" s="17" t="inlineStr">
         <is>
@@ -6018,16 +6018,16 @@
         <v>1739</v>
       </c>
       <c r="D6" s="22" t="n">
-        <v>0.3592</v>
+        <v>0.3598</v>
       </c>
       <c r="E6" s="22" t="n">
-        <v>0.3336</v>
+        <v>0.3226</v>
       </c>
       <c r="F6" s="22" t="n">
-        <v>0.1902</v>
+        <v>0.2088</v>
       </c>
       <c r="G6" s="22" t="n">
-        <v>0.117</v>
+        <v>0.1088</v>
       </c>
       <c r="H6" s="20" t="inlineStr">
         <is>
@@ -6046,16 +6046,16 @@
         <v>1687</v>
       </c>
       <c r="N6" s="22" t="n">
-        <v>0.33</v>
+        <v>0.339</v>
       </c>
       <c r="O6" s="22" t="n">
-        <v>0.3552</v>
+        <v>0.3432</v>
       </c>
       <c r="P6" s="22" t="n">
-        <v>0.2122</v>
+        <v>0.217</v>
       </c>
       <c r="Q6" s="22" t="n">
-        <v>0.1025999999999999</v>
+        <v>0.1008</v>
       </c>
       <c r="R6" s="20" t="inlineStr">
         <is>
@@ -6074,16 +6074,16 @@
         <v>1734</v>
       </c>
       <c r="X6" s="22" t="n">
-        <v>0.2862</v>
+        <v>0.2812</v>
       </c>
       <c r="Y6" s="22" t="n">
-        <v>0.269</v>
+        <v>0.2804</v>
       </c>
       <c r="Z6" s="22" t="n">
-        <v>0.2456</v>
+        <v>0.2406</v>
       </c>
       <c r="AA6" s="22" t="n">
-        <v>0.1992</v>
+        <v>0.1978</v>
       </c>
       <c r="AB6" s="20" t="inlineStr">
         <is>
@@ -6102,16 +6102,16 @@
         <v>1821</v>
       </c>
       <c r="AH6" s="22" t="n">
-        <v>0.3534</v>
+        <v>0.3636</v>
       </c>
       <c r="AI6" s="22" t="n">
-        <v>0.404</v>
+        <v>0.3928</v>
       </c>
       <c r="AJ6" s="22" t="n">
-        <v>0.1758</v>
+        <v>0.1806</v>
       </c>
       <c r="AK6" s="22" t="n">
-        <v>0.06680000000000003</v>
+        <v>0.06300000000000008</v>
       </c>
       <c r="AL6" s="20" t="inlineStr">
         <is>
@@ -6132,16 +6132,16 @@
         <v>1579</v>
       </c>
       <c r="D7" s="25" t="n">
-        <v>0.114</v>
+        <v>0.1188</v>
       </c>
       <c r="E7" s="25" t="n">
-        <v>0.202</v>
+        <v>0.2122</v>
       </c>
       <c r="F7" s="25" t="n">
-        <v>0.3382</v>
+        <v>0.3232</v>
       </c>
       <c r="G7" s="25" t="n">
-        <v>0.3457999999999999</v>
+        <v>0.3458000000000001</v>
       </c>
       <c r="H7" s="26" t="inlineStr">
         <is>
@@ -6160,16 +6160,16 @@
         <v>1551</v>
       </c>
       <c r="N7" s="25" t="n">
-        <v>0.1026</v>
+        <v>0.09959999999999999</v>
       </c>
       <c r="O7" s="25" t="n">
-        <v>0.205</v>
+        <v>0.2056</v>
       </c>
       <c r="P7" s="25" t="n">
-        <v>0.3502</v>
+        <v>0.3418</v>
       </c>
       <c r="Q7" s="25" t="n">
-        <v>0.3422</v>
+        <v>0.353</v>
       </c>
       <c r="R7" s="26" t="inlineStr">
         <is>
@@ -6188,16 +6188,16 @@
         <v>1706</v>
       </c>
       <c r="X7" s="25" t="n">
-        <v>0.2698</v>
+        <v>0.2764</v>
       </c>
       <c r="Y7" s="25" t="n">
-        <v>0.2806</v>
+        <v>0.292</v>
       </c>
       <c r="Z7" s="25" t="n">
-        <v>0.259</v>
+        <v>0.2432</v>
       </c>
       <c r="AA7" s="25" t="n">
-        <v>0.1905999999999999</v>
+        <v>0.1884</v>
       </c>
       <c r="AB7" s="26" t="inlineStr">
         <is>
@@ -6216,16 +6216,16 @@
         <v>1611</v>
       </c>
       <c r="AH7" s="25" t="n">
-        <v>0.07340000000000001</v>
+        <v>0.0774</v>
       </c>
       <c r="AI7" s="25" t="n">
-        <v>0.1814</v>
+        <v>0.1824</v>
       </c>
       <c r="AJ7" s="25" t="n">
-        <v>0.4084</v>
+        <v>0.4054</v>
       </c>
       <c r="AK7" s="25" t="n">
-        <v>0.3368</v>
+        <v>0.3348</v>
       </c>
       <c r="AL7" s="26" t="inlineStr">
         <is>
@@ -6246,16 +6246,16 @@
         <v>1556</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>0.0838</v>
+        <v>0.079</v>
       </c>
       <c r="E8" s="29" t="n">
-        <v>0.1578</v>
+        <v>0.1534</v>
       </c>
       <c r="F8" s="29" t="n">
-        <v>0.304</v>
+        <v>0.3076</v>
       </c>
       <c r="G8" s="29" t="n">
-        <v>0.4544</v>
+        <v>0.4600000000000001</v>
       </c>
       <c r="H8" s="30" t="inlineStr">
         <is>
@@ -6274,16 +6274,16 @@
         <v>1475</v>
       </c>
       <c r="N8" s="29" t="n">
-        <v>0.0634</v>
+        <v>0.0684</v>
       </c>
       <c r="O8" s="29" t="n">
-        <v>0.1518</v>
+        <v>0.1528</v>
       </c>
       <c r="P8" s="29" t="n">
-        <v>0.2884</v>
+        <v>0.3016</v>
       </c>
       <c r="Q8" s="29" t="n">
-        <v>0.4964</v>
+        <v>0.4772</v>
       </c>
       <c r="R8" s="30" t="inlineStr">
         <is>
@@ -6302,16 +6302,16 @@
         <v>1637</v>
       </c>
       <c r="X8" s="29" t="n">
-        <v>0.1094</v>
+        <v>0.0992</v>
       </c>
       <c r="Y8" s="29" t="n">
-        <v>0.1734</v>
+        <v>0.1714</v>
       </c>
       <c r="Z8" s="29" t="n">
-        <v>0.2608</v>
+        <v>0.2728</v>
       </c>
       <c r="AA8" s="29" t="n">
-        <v>0.4564000000000001</v>
+        <v>0.4566000000000001</v>
       </c>
       <c r="AB8" s="30" t="inlineStr">
         <is>
@@ -6330,16 +6330,16 @@
         <v>1509</v>
       </c>
       <c r="AH8" s="29" t="n">
-        <v>0.0326</v>
+        <v>0.032</v>
       </c>
       <c r="AI8" s="29" t="n">
-        <v>0.1042</v>
+        <v>0.103</v>
       </c>
       <c r="AJ8" s="29" t="n">
-        <v>0.299</v>
+        <v>0.2938</v>
       </c>
       <c r="AK8" s="29" t="n">
-        <v>0.5642</v>
+        <v>0.5711999999999999</v>
       </c>
       <c r="AL8" s="30" t="inlineStr">
         <is>
@@ -6544,16 +6544,16 @@
         <v>1806</v>
       </c>
       <c r="D13" s="19" t="n">
-        <v>0.5738</v>
+        <v>0.577</v>
       </c>
       <c r="E13" s="19" t="n">
-        <v>0.2678</v>
+        <v>0.2642</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>0.1228</v>
+        <v>0.1186</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>0.03560000000000003</v>
+        <v>0.04020000000000006</v>
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
@@ -6572,16 +6572,16 @@
         <v>1815</v>
       </c>
       <c r="N13" s="19" t="n">
-        <v>0.4496</v>
+        <v>0.4396</v>
       </c>
       <c r="O13" s="19" t="n">
-        <v>0.3458</v>
+        <v>0.3476</v>
       </c>
       <c r="P13" s="19" t="n">
-        <v>0.1478</v>
+        <v>0.1592</v>
       </c>
       <c r="Q13" s="19" t="n">
-        <v>0.05680000000000002</v>
+        <v>0.05359999999999998</v>
       </c>
       <c r="R13" s="17" t="inlineStr">
         <is>
@@ -6600,16 +6600,16 @@
         <v>1776</v>
       </c>
       <c r="X13" s="19" t="n">
-        <v>0.445</v>
+        <v>0.4542</v>
       </c>
       <c r="Y13" s="19" t="n">
-        <v>0.2894</v>
+        <v>0.2944</v>
       </c>
       <c r="Z13" s="19" t="n">
-        <v>0.188</v>
+        <v>0.177</v>
       </c>
       <c r="AA13" s="19" t="n">
-        <v>0.07759999999999995</v>
+        <v>0.07440000000000008</v>
       </c>
       <c r="AB13" s="17" t="inlineStr">
         <is>
@@ -6628,16 +6628,16 @@
         <v>1959</v>
       </c>
       <c r="AH13" s="19" t="n">
-        <v>0.781</v>
+        <v>0.7824</v>
       </c>
       <c r="AI13" s="19" t="n">
-        <v>0.176</v>
+        <v>0.169</v>
       </c>
       <c r="AJ13" s="19" t="n">
-        <v>0.0358</v>
+        <v>0.0414</v>
       </c>
       <c r="AK13" s="19" t="n">
-        <v>0.007199999999999984</v>
+        <v>0.007200000000000005</v>
       </c>
       <c r="AL13" s="17" t="inlineStr">
         <is>
@@ -6658,16 +6658,16 @@
         <v>1730</v>
       </c>
       <c r="D14" s="22" t="n">
-        <v>0.2084</v>
+        <v>0.2086</v>
       </c>
       <c r="E14" s="22" t="n">
-        <v>0.339</v>
+        <v>0.3348</v>
       </c>
       <c r="F14" s="22" t="n">
-        <v>0.313</v>
+        <v>0.318</v>
       </c>
       <c r="G14" s="22" t="n">
-        <v>0.1395999999999999</v>
+        <v>0.1386</v>
       </c>
       <c r="H14" s="20" t="inlineStr">
         <is>
@@ -6686,16 +6686,16 @@
         <v>1820</v>
       </c>
       <c r="N14" s="22" t="n">
-        <v>0.4262</v>
+        <v>0.4376</v>
       </c>
       <c r="O14" s="22" t="n">
-        <v>0.3486</v>
+        <v>0.3474</v>
       </c>
       <c r="P14" s="22" t="n">
-        <v>0.1592</v>
+        <v>0.1546</v>
       </c>
       <c r="Q14" s="22" t="n">
-        <v>0.06599999999999995</v>
+        <v>0.06040000000000004</v>
       </c>
       <c r="R14" s="20" t="inlineStr">
         <is>
@@ -6714,16 +6714,16 @@
         <v>1756</v>
       </c>
       <c r="X14" s="22" t="n">
-        <v>0.3214</v>
+        <v>0.328</v>
       </c>
       <c r="Y14" s="22" t="n">
-        <v>0.323</v>
+        <v>0.3312</v>
       </c>
       <c r="Z14" s="22" t="n">
-        <v>0.2382</v>
+        <v>0.2314</v>
       </c>
       <c r="AA14" s="22" t="n">
-        <v>0.1174</v>
+        <v>0.1093999999999999</v>
       </c>
       <c r="AB14" s="20" t="inlineStr">
         <is>
@@ -6742,16 +6742,16 @@
         <v>1745</v>
       </c>
       <c r="AH14" s="22" t="n">
-        <v>0.1584</v>
+        <v>0.157</v>
       </c>
       <c r="AI14" s="22" t="n">
-        <v>0.499</v>
+        <v>0.5104</v>
       </c>
       <c r="AJ14" s="22" t="n">
-        <v>0.2406</v>
+        <v>0.236</v>
       </c>
       <c r="AK14" s="22" t="n">
-        <v>0.102</v>
+        <v>0.09660000000000002</v>
       </c>
       <c r="AL14" s="20" t="inlineStr">
         <is>
@@ -6772,16 +6772,16 @@
         <v>1662</v>
       </c>
       <c r="D15" s="25" t="n">
-        <v>0.1914</v>
+        <v>0.181</v>
       </c>
       <c r="E15" s="25" t="n">
-        <v>0.3006</v>
+        <v>0.314</v>
       </c>
       <c r="F15" s="25" t="n">
-        <v>0.3406</v>
+        <v>0.3452</v>
       </c>
       <c r="G15" s="25" t="n">
-        <v>0.1674</v>
+        <v>0.1597999999999999</v>
       </c>
       <c r="H15" s="26" t="inlineStr">
         <is>
@@ -6800,16 +6800,16 @@
         <v>1625</v>
       </c>
       <c r="N15" s="25" t="n">
-        <v>0.074</v>
+        <v>0.0746</v>
       </c>
       <c r="O15" s="25" t="n">
-        <v>0.1778</v>
+        <v>0.18</v>
       </c>
       <c r="P15" s="25" t="n">
-        <v>0.4084</v>
+        <v>0.39</v>
       </c>
       <c r="Q15" s="25" t="n">
-        <v>0.3398</v>
+        <v>0.3554</v>
       </c>
       <c r="R15" s="26" t="inlineStr">
         <is>
@@ -6828,16 +6828,16 @@
         <v>1675</v>
       </c>
       <c r="X15" s="25" t="n">
-        <v>0.1806</v>
+        <v>0.17</v>
       </c>
       <c r="Y15" s="25" t="n">
-        <v>0.2822</v>
+        <v>0.262</v>
       </c>
       <c r="Z15" s="25" t="n">
-        <v>0.3304</v>
+        <v>0.3562</v>
       </c>
       <c r="AA15" s="25" t="n">
-        <v>0.2068</v>
+        <v>0.2117999999999999</v>
       </c>
       <c r="AB15" s="26" t="inlineStr">
         <is>
@@ -6856,13 +6856,13 @@
         <v>1578</v>
       </c>
       <c r="AH15" s="25" t="n">
-        <v>0.0412</v>
+        <v>0.0386</v>
       </c>
       <c r="AI15" s="25" t="n">
-        <v>0.197</v>
+        <v>0.1856</v>
       </c>
       <c r="AJ15" s="25" t="n">
-        <v>0.3856</v>
+        <v>0.3996</v>
       </c>
       <c r="AK15" s="25" t="n">
         <v>0.3762</v>
@@ -6886,16 +6886,16 @@
         <v>1491</v>
       </c>
       <c r="D16" s="29" t="n">
-        <v>0.0264</v>
+        <v>0.0334</v>
       </c>
       <c r="E16" s="29" t="n">
-        <v>0.0926</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="F16" s="29" t="n">
-        <v>0.2236</v>
+        <v>0.2182</v>
       </c>
       <c r="G16" s="29" t="n">
-        <v>0.6574</v>
+        <v>0.6614</v>
       </c>
       <c r="H16" s="30" t="inlineStr">
         <is>
@@ -6914,16 +6914,16 @@
         <v>1579</v>
       </c>
       <c r="N16" s="29" t="n">
-        <v>0.0502</v>
+        <v>0.0482</v>
       </c>
       <c r="O16" s="29" t="n">
-        <v>0.1278</v>
+        <v>0.125</v>
       </c>
       <c r="P16" s="29" t="n">
-        <v>0.2846</v>
+        <v>0.2962</v>
       </c>
       <c r="Q16" s="29" t="n">
-        <v>0.5373999999999999</v>
+        <v>0.5306</v>
       </c>
       <c r="R16" s="30" t="inlineStr">
         <is>
@@ -6942,16 +6942,16 @@
         <v>1547</v>
       </c>
       <c r="X16" s="29" t="n">
-        <v>0.053</v>
+        <v>0.0478</v>
       </c>
       <c r="Y16" s="29" t="n">
-        <v>0.1054</v>
+        <v>0.1124</v>
       </c>
       <c r="Z16" s="29" t="n">
-        <v>0.2434</v>
+        <v>0.2354</v>
       </c>
       <c r="AA16" s="29" t="n">
-        <v>0.5981999999999998</v>
+        <v>0.6044</v>
       </c>
       <c r="AB16" s="30" t="inlineStr">
         <is>
@@ -6970,16 +6970,16 @@
         <v>1512</v>
       </c>
       <c r="AH16" s="29" t="n">
-        <v>0.0194</v>
+        <v>0.022</v>
       </c>
       <c r="AI16" s="29" t="n">
-        <v>0.128</v>
+        <v>0.135</v>
       </c>
       <c r="AJ16" s="29" t="n">
-        <v>0.338</v>
+        <v>0.323</v>
       </c>
       <c r="AK16" s="29" t="n">
-        <v>0.5145999999999999</v>
+        <v>0.52</v>
       </c>
       <c r="AL16" s="30" t="inlineStr">
         <is>
@@ -7184,16 +7184,16 @@
         <v>1923</v>
       </c>
       <c r="D21" s="19" t="n">
-        <v>0.6088</v>
+        <v>0.6094000000000001</v>
       </c>
       <c r="E21" s="19" t="n">
-        <v>0.248</v>
+        <v>0.259</v>
       </c>
       <c r="F21" s="19" t="n">
-        <v>0.1076</v>
+        <v>0.09619999999999999</v>
       </c>
       <c r="G21" s="19" t="n">
-        <v>0.03559999999999999</v>
+        <v>0.03539999999999995</v>
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
@@ -7212,16 +7212,16 @@
         <v>1925</v>
       </c>
       <c r="N21" s="19" t="n">
-        <v>0.6844</v>
+        <v>0.6929999999999999</v>
       </c>
       <c r="O21" s="19" t="n">
-        <v>0.214</v>
+        <v>0.2066</v>
       </c>
       <c r="P21" s="19" t="n">
-        <v>0.0752</v>
+        <v>0.07340000000000001</v>
       </c>
       <c r="Q21" s="19" t="n">
-        <v>0.02639999999999999</v>
+        <v>0.02700000000000004</v>
       </c>
       <c r="R21" s="17" t="inlineStr">
         <is>
@@ -7240,16 +7240,16 @@
         <v>1813</v>
       </c>
       <c r="X21" s="19" t="n">
-        <v>0.4466</v>
+        <v>0.4526</v>
       </c>
       <c r="Y21" s="19" t="n">
-        <v>0.289</v>
+        <v>0.2916</v>
       </c>
       <c r="Z21" s="19" t="n">
-        <v>0.168</v>
+        <v>0.1632</v>
       </c>
       <c r="AA21" s="19" t="n">
-        <v>0.09640000000000001</v>
+        <v>0.09259999999999996</v>
       </c>
       <c r="AB21" s="17" t="inlineStr">
         <is>
@@ -7268,16 +7268,16 @@
         <v>1890</v>
       </c>
       <c r="AH21" s="19" t="n">
-        <v>0.5648</v>
+        <v>0.5698</v>
       </c>
       <c r="AI21" s="19" t="n">
-        <v>0.2808</v>
+        <v>0.28</v>
       </c>
       <c r="AJ21" s="19" t="n">
-        <v>0.1272</v>
+        <v>0.1238</v>
       </c>
       <c r="AK21" s="19" t="n">
-        <v>0.02720000000000003</v>
+        <v>0.02640000000000001</v>
       </c>
       <c r="AL21" s="17" t="inlineStr">
         <is>
@@ -7298,16 +7298,16 @@
         <v>1779</v>
       </c>
       <c r="D22" s="22" t="n">
-        <v>0.2364</v>
+        <v>0.2434</v>
       </c>
       <c r="E22" s="22" t="n">
-        <v>0.3638</v>
+        <v>0.378</v>
       </c>
       <c r="F22" s="22" t="n">
-        <v>0.264</v>
+        <v>0.2528</v>
       </c>
       <c r="G22" s="22" t="n">
-        <v>0.1358</v>
+        <v>0.1257999999999999</v>
       </c>
       <c r="H22" s="20" t="inlineStr">
         <is>
@@ -7326,16 +7326,16 @@
         <v>1707</v>
       </c>
       <c r="N22" s="22" t="n">
-        <v>0.1496</v>
+        <v>0.1504</v>
       </c>
       <c r="O22" s="22" t="n">
-        <v>0.3412</v>
+        <v>0.3416</v>
       </c>
       <c r="P22" s="22" t="n">
-        <v>0.304</v>
+        <v>0.3038</v>
       </c>
       <c r="Q22" s="22" t="n">
-        <v>0.2052000000000001</v>
+        <v>0.2042</v>
       </c>
       <c r="R22" s="20" t="inlineStr">
         <is>
@@ -7357,13 +7357,13 @@
         <v>0.3138</v>
       </c>
       <c r="Y22" s="22" t="n">
-        <v>0.3082</v>
+        <v>0.3132</v>
       </c>
       <c r="Z22" s="22" t="n">
-        <v>0.233</v>
+        <v>0.221</v>
       </c>
       <c r="AA22" s="22" t="n">
-        <v>0.1449999999999999</v>
+        <v>0.1519999999999999</v>
       </c>
       <c r="AB22" s="20" t="inlineStr">
         <is>
@@ -7382,16 +7382,16 @@
         <v>1778</v>
       </c>
       <c r="AH22" s="22" t="n">
-        <v>0.2998</v>
+        <v>0.2874</v>
       </c>
       <c r="AI22" s="22" t="n">
-        <v>0.3852</v>
+        <v>0.3922</v>
       </c>
       <c r="AJ22" s="22" t="n">
-        <v>0.2352</v>
+        <v>0.2428</v>
       </c>
       <c r="AK22" s="22" t="n">
-        <v>0.07979999999999995</v>
+        <v>0.07760000000000003</v>
       </c>
       <c r="AL22" s="20" t="inlineStr">
         <is>
@@ -7412,16 +7412,16 @@
         <v>1692</v>
       </c>
       <c r="D23" s="25" t="n">
-        <v>0.1032</v>
+        <v>0.1044</v>
       </c>
       <c r="E23" s="25" t="n">
-        <v>0.2478</v>
+        <v>0.2328</v>
       </c>
       <c r="F23" s="25" t="n">
-        <v>0.3522</v>
+        <v>0.374</v>
       </c>
       <c r="G23" s="25" t="n">
-        <v>0.2968</v>
+        <v>0.2887999999999999</v>
       </c>
       <c r="H23" s="26" t="inlineStr">
         <is>
@@ -7440,16 +7440,16 @@
         <v>1663</v>
       </c>
       <c r="N23" s="25" t="n">
-        <v>0.1104</v>
+        <v>0.1024</v>
       </c>
       <c r="O23" s="25" t="n">
-        <v>0.281</v>
+        <v>0.2776</v>
       </c>
       <c r="P23" s="25" t="n">
-        <v>0.337</v>
+        <v>0.345</v>
       </c>
       <c r="Q23" s="25" t="n">
-        <v>0.2715999999999999</v>
+        <v>0.2749999999999999</v>
       </c>
       <c r="R23" s="26" t="inlineStr">
         <is>
@@ -7468,16 +7468,16 @@
         <v>1671</v>
       </c>
       <c r="X23" s="25" t="n">
-        <v>0.1396</v>
+        <v>0.1364</v>
       </c>
       <c r="Y23" s="25" t="n">
-        <v>0.2202</v>
+        <v>0.217</v>
       </c>
       <c r="Z23" s="25" t="n">
-        <v>0.3144</v>
+        <v>0.3214</v>
       </c>
       <c r="AA23" s="25" t="n">
-        <v>0.3258000000000001</v>
+        <v>0.3252</v>
       </c>
       <c r="AB23" s="26" t="inlineStr">
         <is>
@@ -7496,16 +7496,16 @@
         <v>1673</v>
       </c>
       <c r="AH23" s="25" t="n">
-        <v>0.1148</v>
+        <v>0.1224</v>
       </c>
       <c r="AI23" s="25" t="n">
-        <v>0.2612</v>
+        <v>0.2556</v>
       </c>
       <c r="AJ23" s="25" t="n">
-        <v>0.4204</v>
+        <v>0.4186</v>
       </c>
       <c r="AK23" s="25" t="n">
-        <v>0.2036</v>
+        <v>0.2034000000000001</v>
       </c>
       <c r="AL23" s="26" t="inlineStr">
         <is>
@@ -7526,16 +7526,16 @@
         <v>1615</v>
       </c>
       <c r="D24" s="29" t="n">
-        <v>0.0516</v>
+        <v>0.0428</v>
       </c>
       <c r="E24" s="29" t="n">
-        <v>0.1404</v>
+        <v>0.1302</v>
       </c>
       <c r="F24" s="29" t="n">
-        <v>0.2762</v>
+        <v>0.277</v>
       </c>
       <c r="G24" s="29" t="n">
-        <v>0.5318000000000001</v>
+        <v>0.55</v>
       </c>
       <c r="H24" s="30" t="inlineStr">
         <is>
@@ -7554,16 +7554,16 @@
         <v>1607</v>
       </c>
       <c r="N24" s="29" t="n">
-        <v>0.0556</v>
+        <v>0.0542</v>
       </c>
       <c r="O24" s="29" t="n">
-        <v>0.1638</v>
+        <v>0.1742</v>
       </c>
       <c r="P24" s="29" t="n">
-        <v>0.2838</v>
+        <v>0.2778</v>
       </c>
       <c r="Q24" s="29" t="n">
-        <v>0.4968</v>
+        <v>0.4938</v>
       </c>
       <c r="R24" s="30" t="inlineStr">
         <is>
@@ -7582,16 +7582,16 @@
         <v>1620</v>
       </c>
       <c r="X24" s="29" t="n">
-        <v>0.1</v>
+        <v>0.09719999999999999</v>
       </c>
       <c r="Y24" s="29" t="n">
-        <v>0.1826</v>
+        <v>0.1782</v>
       </c>
       <c r="Z24" s="29" t="n">
-        <v>0.2846</v>
+        <v>0.2944</v>
       </c>
       <c r="AA24" s="29" t="n">
-        <v>0.4328</v>
+        <v>0.4302</v>
       </c>
       <c r="AB24" s="30" t="inlineStr">
         <is>
@@ -7610,16 +7610,16 @@
         <v>1508</v>
       </c>
       <c r="AH24" s="29" t="n">
-        <v>0.0206</v>
+        <v>0.0204</v>
       </c>
       <c r="AI24" s="29" t="n">
-        <v>0.0728</v>
+        <v>0.0722</v>
       </c>
       <c r="AJ24" s="29" t="n">
-        <v>0.2172</v>
+        <v>0.2148</v>
       </c>
       <c r="AK24" s="29" t="n">
-        <v>0.6894</v>
+        <v>0.6926</v>
       </c>
       <c r="AL24" s="30" t="inlineStr">
         <is>
@@ -7758,16 +7758,16 @@
           <t>Switzerland</t>
         </is>
       </c>
-      <c r="D4" s="34" t="n">
+      <c r="D4" s="35" t="n">
+        <v>0.366</v>
+      </c>
+      <c r="E4" s="33" t="inlineStr">
+        <is>
+          <t>South Korea</t>
+        </is>
+      </c>
+      <c r="F4" s="34" t="n">
         <v>0.376</v>
-      </c>
-      <c r="E4" s="33" t="inlineStr">
-        <is>
-          <t>South Korea</t>
-        </is>
-      </c>
-      <c r="F4" s="35" t="n">
-        <v>0.366</v>
       </c>
       <c r="G4" s="36" t="inlineStr">
         <is>
@@ -7791,16 +7791,16 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="D5" s="35" t="n">
+        <v>0.303</v>
+      </c>
+      <c r="E5" s="33" t="inlineStr">
+        <is>
+          <t>Brazil</t>
+        </is>
+      </c>
+      <c r="F5" s="34" t="n">
         <v>0.464</v>
-      </c>
-      <c r="E5" s="33" t="inlineStr">
-        <is>
-          <t>Brazil</t>
-        </is>
-      </c>
-      <c r="F5" s="35" t="n">
-        <v>0.303</v>
       </c>
       <c r="G5" s="36" t="inlineStr">
         <is>
@@ -7825,15 +7825,15 @@
         </is>
       </c>
       <c r="D6" s="34" t="n">
-        <v>0.551</v>
+        <v>0.518</v>
       </c>
       <c r="E6" s="33" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="F6" s="35" t="n">
-        <v>0.239</v>
+        <v>0.263</v>
       </c>
       <c r="G6" s="36" t="inlineStr">
         <is>
@@ -7857,20 +7857,20 @@
           <t>Germany</t>
         </is>
       </c>
-      <c r="D7" s="34" t="n">
-        <v>0.382</v>
+      <c r="D7" s="35" t="n">
+        <v>0.358</v>
       </c>
       <c r="E7" s="33" t="inlineStr">
         <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="F7" s="35" t="n">
-        <v>0.362</v>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="F7" s="34" t="n">
+        <v>0.389</v>
       </c>
       <c r="G7" s="36" t="inlineStr">
         <is>
-          <t>→ Japan</t>
+          <t>→ Netherlands</t>
         </is>
       </c>
     </row>
@@ -8089,15 +8089,15 @@
         </is>
       </c>
       <c r="D14" s="34" t="n">
-        <v>0.468</v>
+        <v>0.508</v>
       </c>
       <c r="E14" s="33" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="F14" s="35" t="n">
-        <v>0.301</v>
+        <v>0.271</v>
       </c>
       <c r="G14" s="36" t="inlineStr">
         <is>
@@ -8287,16 +8287,16 @@
           <t>Brazil</t>
         </is>
       </c>
-      <c r="D21" s="34" t="n">
+      <c r="D21" s="35" t="n">
+        <v>0.344</v>
+      </c>
+      <c r="E21" s="39" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="F21" s="34" t="n">
         <v>0.408</v>
-      </c>
-      <c r="E21" s="39" t="inlineStr">
-        <is>
-          <t>Morocco</t>
-        </is>
-      </c>
-      <c r="F21" s="35" t="n">
-        <v>0.344</v>
       </c>
       <c r="G21" s="40" t="inlineStr">
         <is>
@@ -8317,23 +8317,23 @@
       </c>
       <c r="C22" s="39" t="inlineStr">
         <is>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="n">
+        <v>0.377</v>
+      </c>
+      <c r="E22" s="39" t="inlineStr">
+        <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="D22" s="34" t="n">
-        <v>0.371</v>
-      </c>
-      <c r="E22" s="39" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="F22" s="34" t="n">
-        <v>0.371</v>
+      <c r="F22" s="35" t="n">
+        <v>0.366</v>
       </c>
       <c r="G22" s="40" t="inlineStr">
         <is>
-          <t>→ Japan</t>
+          <t>→ Netherlands</t>
         </is>
       </c>
     </row>
@@ -8353,16 +8353,16 @@
           <t>Belgium</t>
         </is>
       </c>
-      <c r="D23" s="34" t="n">
+      <c r="D23" s="35" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="E23" s="39" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="F23" s="34" t="n">
         <v>0.594</v>
-      </c>
-      <c r="E23" s="39" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="F23" s="35" t="n">
-        <v>0.207</v>
       </c>
       <c r="G23" s="40" t="inlineStr">
         <is>
@@ -8386,16 +8386,16 @@
           <t>France</t>
         </is>
       </c>
-      <c r="D24" s="34" t="n">
+      <c r="D24" s="35" t="n">
+        <v>0.369</v>
+      </c>
+      <c r="E24" s="39" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="F24" s="34" t="n">
         <v>0.373</v>
-      </c>
-      <c r="E24" s="39" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="F24" s="35" t="n">
-        <v>0.369</v>
       </c>
       <c r="G24" s="40" t="inlineStr">
         <is>
@@ -8419,16 +8419,16 @@
           <t>Portugal</t>
         </is>
       </c>
-      <c r="D25" s="34" t="n">
+      <c r="D25" s="35" t="n">
+        <v>0.301</v>
+      </c>
+      <c r="E25" s="39" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="F25" s="34" t="n">
         <v>0.468</v>
-      </c>
-      <c r="E25" s="39" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="F25" s="35" t="n">
-        <v>0.301</v>
       </c>
       <c r="G25" s="40" t="inlineStr">
         <is>
@@ -8452,16 +8452,16 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="D26" s="34" t="n">
+      <c r="D26" s="35" t="n">
+        <v>0.276</v>
+      </c>
+      <c r="E26" s="39" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="F26" s="34" t="n">
         <v>0.501</v>
-      </c>
-      <c r="E26" s="39" t="inlineStr">
-        <is>
-          <t>Morocco</t>
-        </is>
-      </c>
-      <c r="F26" s="35" t="n">
-        <v>0.276</v>
       </c>
       <c r="G26" s="40" t="inlineStr">
         <is>
@@ -8485,16 +8485,16 @@
           <t>Belgium</t>
         </is>
       </c>
-      <c r="D27" s="34" t="n">
+      <c r="D27" s="35" t="n">
+        <v>0.207</v>
+      </c>
+      <c r="E27" s="39" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="F27" s="34" t="n">
         <v>0.594</v>
-      </c>
-      <c r="E27" s="39" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="F27" s="35" t="n">
-        <v>0.207</v>
       </c>
       <c r="G27" s="40" t="inlineStr">
         <is>
@@ -8519,16 +8519,16 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="D29" s="34" t="n">
+      <c r="D29" s="35" t="n">
+        <v>0.289</v>
+      </c>
+      <c r="E29" s="43" t="inlineStr">
+        <is>
+          <t>Morocco</t>
+        </is>
+      </c>
+      <c r="F29" s="34" t="n">
         <v>0.483</v>
-      </c>
-      <c r="E29" s="43" t="inlineStr">
-        <is>
-          <t>Morocco</t>
-        </is>
-      </c>
-      <c r="F29" s="35" t="n">
-        <v>0.289</v>
       </c>
       <c r="G29" s="44" t="inlineStr">
         <is>
@@ -8549,19 +8549,19 @@
       </c>
       <c r="C30" s="43" t="inlineStr">
         <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D30" s="34" t="n">
-        <v>0.55</v>
+          <t>Netherlands</t>
+        </is>
+      </c>
+      <c r="D30" s="35" t="n">
+        <v>0.244</v>
       </c>
       <c r="E30" s="43" t="inlineStr">
         <is>
           <t>Spain</t>
         </is>
       </c>
-      <c r="F30" s="35" t="n">
-        <v>0.24</v>
+      <c r="F30" s="34" t="n">
+        <v>0.544</v>
       </c>
       <c r="G30" s="44" t="inlineStr">
         <is>
@@ -8618,16 +8618,16 @@
           <t>Morocco</t>
         </is>
       </c>
-      <c r="D32" s="34" t="n">
+      <c r="D32" s="35" t="n">
+        <v>0.272</v>
+      </c>
+      <c r="E32" s="43" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="F32" s="34" t="n">
         <v>0.507</v>
-      </c>
-      <c r="E32" s="43" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="F32" s="35" t="n">
-        <v>0.272</v>
       </c>
       <c r="G32" s="44" t="inlineStr">
         <is>
@@ -8652,16 +8652,16 @@
           <t>Morocco</t>
         </is>
       </c>
-      <c r="D34" s="34" t="n">
+      <c r="D34" s="35" t="n">
+        <v>0.272</v>
+      </c>
+      <c r="E34" s="47" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="F34" s="34" t="n">
         <v>0.507</v>
-      </c>
-      <c r="E34" s="47" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="F34" s="35" t="n">
-        <v>0.272</v>
       </c>
       <c r="G34" s="48" t="inlineStr">
         <is>
@@ -8685,16 +8685,16 @@
           <t>Argentina</t>
         </is>
       </c>
-      <c r="D35" s="34" t="n">
+      <c r="D35" s="35" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="E35" s="47" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="F35" s="34" t="n">
         <v>0.414</v>
-      </c>
-      <c r="E35" s="47" t="inlineStr">
-        <is>
-          <t>Spain</t>
-        </is>
-      </c>
-      <c r="F35" s="35" t="n">
-        <v>0.34</v>
       </c>
       <c r="G35" s="48" t="inlineStr">
         <is>
@@ -8750,7 +8750,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G50"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8824,11 +8824,11 @@
         <v>0.2285</v>
       </c>
       <c r="E3" s="55" t="n">
-        <v>0.2316</v>
+        <v>0.2321</v>
       </c>
       <c r="F3" s="56" t="inlineStr">
         <is>
-          <t>↑ 0.3%</t>
+          <t>↑ 0.4%</t>
         </is>
       </c>
       <c r="G3" s="57" t="inlineStr">
@@ -8855,16 +8855,16 @@
         <v>0.1168</v>
       </c>
       <c r="E4" s="61" t="n">
-        <v>0.1469</v>
+        <v>0.1443</v>
       </c>
       <c r="F4" s="62" t="inlineStr">
         <is>
-          <t>↑ 3.0%</t>
+          <t>↑ 2.8%</t>
         </is>
       </c>
       <c r="G4" s="63" t="inlineStr">
         <is>
-          <t>██████████████████████░░░░░░░░░░░░░░░░░░░░░░░</t>
+          <t>█████████████████████░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
       </c>
     </row>
@@ -8886,11 +8886,11 @@
         <v>0.11</v>
       </c>
       <c r="E5" s="67" t="n">
-        <v>0.1415</v>
+        <v>0.1413</v>
       </c>
       <c r="F5" s="68" t="inlineStr">
         <is>
-          <t>↑ 3.2%</t>
+          <t>↑ 3.1%</t>
         </is>
       </c>
       <c r="G5" s="69" t="inlineStr">
@@ -8917,11 +8917,11 @@
         <v>0.08500000000000001</v>
       </c>
       <c r="E6" s="70" t="n">
-        <v>0.0852</v>
+        <v>0.08560000000000001</v>
       </c>
       <c r="F6" s="71" t="inlineStr">
         <is>
-          <t>→ 0.0%</t>
+          <t>→ 0.1%</t>
         </is>
       </c>
       <c r="G6" s="72" t="inlineStr">
@@ -8948,11 +8948,11 @@
         <v>0.0702</v>
       </c>
       <c r="E7" s="73" t="n">
-        <v>0.07389999999999999</v>
+        <v>0.07539999999999999</v>
       </c>
       <c r="F7" s="74" t="inlineStr">
         <is>
-          <t>↑ 0.4%</t>
+          <t>↑ 0.5%</t>
         </is>
       </c>
       <c r="G7" s="75" t="inlineStr">
@@ -8967,7 +8967,7 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -8976,14 +8976,14 @@
         </is>
       </c>
       <c r="D8" s="70" t="n">
-        <v>0.0313</v>
+        <v>0.07480000000000001</v>
       </c>
       <c r="E8" s="70" t="n">
-        <v>0.0428</v>
+        <v>0.043</v>
       </c>
       <c r="F8" s="76" t="inlineStr">
         <is>
-          <t>↑ 1.2%</t>
+          <t>↓ 3.2%</t>
         </is>
       </c>
       <c r="G8" s="72" t="inlineStr">
@@ -8998,7 +8998,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -9007,14 +9007,14 @@
         </is>
       </c>
       <c r="D9" s="73" t="n">
-        <v>0.07480000000000001</v>
+        <v>0.0313</v>
       </c>
       <c r="E9" s="73" t="n">
-        <v>0.0428</v>
-      </c>
-      <c r="F9" s="77" t="inlineStr">
-        <is>
-          <t>↓ 3.2%</t>
+        <v>0.0416</v>
+      </c>
+      <c r="F9" s="74" t="inlineStr">
+        <is>
+          <t>↑ 1.0%</t>
         </is>
       </c>
       <c r="G9" s="75" t="inlineStr">
@@ -9041,7 +9041,7 @@
         <v>0.0334</v>
       </c>
       <c r="E10" s="70" t="n">
-        <v>0.0314</v>
+        <v>0.0318</v>
       </c>
       <c r="F10" s="71" t="inlineStr">
         <is>
@@ -9072,11 +9072,11 @@
         <v>0.0199</v>
       </c>
       <c r="E11" s="73" t="n">
-        <v>0.0302</v>
+        <v>0.0307</v>
       </c>
       <c r="F11" s="74" t="inlineStr">
         <is>
-          <t>↑ 1.0%</t>
+          <t>↑ 1.1%</t>
         </is>
       </c>
       <c r="G11" s="75" t="inlineStr">
@@ -9103,9 +9103,9 @@
         <v>0.0193</v>
       </c>
       <c r="E12" s="70" t="n">
-        <v>0.024</v>
-      </c>
-      <c r="F12" s="76" t="inlineStr">
+        <v>0.0243</v>
+      </c>
+      <c r="F12" s="77" t="inlineStr">
         <is>
           <t>↑ 0.5%</t>
         </is>
@@ -9134,9 +9134,9 @@
         <v>0.0229</v>
       </c>
       <c r="E13" s="73" t="n">
-        <v>0.0192</v>
-      </c>
-      <c r="F13" s="77" t="inlineStr">
+        <v>0.0187</v>
+      </c>
+      <c r="F13" s="78" t="inlineStr">
         <is>
           <t>↓ 0.4%</t>
         </is>
@@ -9165,11 +9165,11 @@
         <v>0.018</v>
       </c>
       <c r="E14" s="70" t="n">
-        <v>0.017</v>
+        <v>0.0182</v>
       </c>
       <c r="F14" s="71" t="inlineStr">
         <is>
-          <t>→ 0.1%</t>
+          <t>→ 0.0%</t>
         </is>
       </c>
       <c r="G14" s="72" t="inlineStr">
@@ -9196,11 +9196,11 @@
         <v>0.0108</v>
       </c>
       <c r="E15" s="73" t="n">
-        <v>0.0169</v>
+        <v>0.0175</v>
       </c>
       <c r="F15" s="74" t="inlineStr">
         <is>
-          <t>↑ 0.6%</t>
+          <t>↑ 0.7%</t>
         </is>
       </c>
       <c r="G15" s="75" t="inlineStr">
@@ -9227,11 +9227,11 @@
         <v>0.011</v>
       </c>
       <c r="E16" s="70" t="n">
-        <v>0.0147</v>
-      </c>
-      <c r="F16" s="76" t="inlineStr">
-        <is>
-          <t>↑ 0.4%</t>
+        <v>0.0144</v>
+      </c>
+      <c r="F16" s="77" t="inlineStr">
+        <is>
+          <t>↑ 0.3%</t>
         </is>
       </c>
       <c r="G16" s="72" t="inlineStr">
@@ -9258,9 +9258,9 @@
         <v>0.0259</v>
       </c>
       <c r="E17" s="73" t="n">
-        <v>0.0111</v>
-      </c>
-      <c r="F17" s="77" t="inlineStr">
+        <v>0.0109</v>
+      </c>
+      <c r="F17" s="78" t="inlineStr">
         <is>
           <t>↓ 1.5%</t>
         </is>
@@ -9289,11 +9289,11 @@
         <v>0.018</v>
       </c>
       <c r="E18" s="70" t="n">
-        <v>0.0098</v>
-      </c>
-      <c r="F18" s="78" t="inlineStr">
-        <is>
-          <t>↓ 0.8%</t>
+        <v>0.0095</v>
+      </c>
+      <c r="F18" s="76" t="inlineStr">
+        <is>
+          <t>↓ 0.9%</t>
         </is>
       </c>
       <c r="G18" s="72" t="inlineStr">
@@ -9320,7 +9320,7 @@
         <v>0.0092</v>
       </c>
       <c r="E19" s="73" t="n">
-        <v>0.009000000000000001</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F19" s="79" t="inlineStr">
         <is>
@@ -9351,11 +9351,11 @@
         <v>0.0098</v>
       </c>
       <c r="E20" s="70" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.007900000000000001</v>
       </c>
       <c r="F20" s="71" t="inlineStr">
         <is>
-          <t>→ 0.1%</t>
+          <t>→ 0.2%</t>
         </is>
       </c>
       <c r="G20" s="72" t="inlineStr">
@@ -9370,23 +9370,23 @@
       </c>
       <c r="B21" s="11" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Iran</t>
         </is>
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Grupo C</t>
+          <t>Grupo G</t>
         </is>
       </c>
       <c r="D21" s="73" t="n">
-        <v>0.0102</v>
+        <v>0.0124</v>
       </c>
       <c r="E21" s="73" t="n">
-        <v>0.005600000000000001</v>
-      </c>
-      <c r="F21" s="77" t="inlineStr">
-        <is>
-          <t>↓ 0.5%</t>
+        <v>0.0061</v>
+      </c>
+      <c r="F21" s="78" t="inlineStr">
+        <is>
+          <t>↓ 0.6%</t>
         </is>
       </c>
       <c r="G21" s="75" t="inlineStr">
@@ -9401,23 +9401,23 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Grupo G</t>
+          <t>Grupo C</t>
         </is>
       </c>
       <c r="D22" s="70" t="n">
-        <v>0.0124</v>
+        <v>0.0102</v>
       </c>
       <c r="E22" s="70" t="n">
-        <v>0.0054</v>
-      </c>
-      <c r="F22" s="78" t="inlineStr">
-        <is>
-          <t>↓ 0.7%</t>
+        <v>0.0058</v>
+      </c>
+      <c r="F22" s="76" t="inlineStr">
+        <is>
+          <t>↓ 0.4%</t>
         </is>
       </c>
       <c r="G22" s="72" t="inlineStr">
@@ -9432,19 +9432,19 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Uruguay</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Grupo H</t>
+          <t>Grupo C</t>
         </is>
       </c>
       <c r="D23" s="73" t="n">
-        <v>0.0039</v>
+        <v>0.0028</v>
       </c>
       <c r="E23" s="73" t="n">
-        <v>0.004500000000000001</v>
+        <v>0.004099999999999999</v>
       </c>
       <c r="F23" s="79" t="inlineStr">
         <is>
@@ -9463,23 +9463,23 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Grupo C</t>
+          <t>Grupo H</t>
         </is>
       </c>
       <c r="D24" s="70" t="n">
-        <v>0.0028</v>
+        <v>0.0039</v>
       </c>
       <c r="E24" s="70" t="n">
-        <v>0.0044</v>
+        <v>0.004</v>
       </c>
       <c r="F24" s="71" t="inlineStr">
         <is>
-          <t>→ 0.2%</t>
+          <t>→ 0.0%</t>
         </is>
       </c>
       <c r="G24" s="72" t="inlineStr">
@@ -9506,9 +9506,9 @@
         <v>0.0086</v>
       </c>
       <c r="E25" s="73" t="n">
-        <v>0.0035</v>
-      </c>
-      <c r="F25" s="77" t="inlineStr">
+        <v>0.0036</v>
+      </c>
+      <c r="F25" s="78" t="inlineStr">
         <is>
           <t>↓ 0.5%</t>
         </is>
@@ -9537,7 +9537,7 @@
         <v>0.0063</v>
       </c>
       <c r="E26" s="70" t="n">
-        <v>0.0033</v>
+        <v>0.0035</v>
       </c>
       <c r="F26" s="71" t="inlineStr">
         <is>
@@ -9568,11 +9568,11 @@
         <v>0.0059</v>
       </c>
       <c r="E27" s="73" t="n">
-        <v>0.0032</v>
+        <v>0.0034</v>
       </c>
       <c r="F27" s="79" t="inlineStr">
         <is>
-          <t>→ 0.3%</t>
+          <t>→ 0.2%</t>
         </is>
       </c>
       <c r="G27" s="75" t="inlineStr">
@@ -9599,7 +9599,7 @@
         <v>0.0049</v>
       </c>
       <c r="E28" s="70" t="n">
-        <v>0.0024</v>
+        <v>0.0026</v>
       </c>
       <c r="F28" s="71" t="inlineStr">
         <is>
@@ -9630,9 +9630,9 @@
         <v>0.0058</v>
       </c>
       <c r="E29" s="73" t="n">
-        <v>0.0024</v>
-      </c>
-      <c r="F29" s="77" t="inlineStr">
+        <v>0.0025</v>
+      </c>
+      <c r="F29" s="78" t="inlineStr">
         <is>
           <t>↓ 0.3%</t>
         </is>
@@ -9723,11 +9723,11 @@
         <v>0.0036</v>
       </c>
       <c r="E32" s="70" t="n">
-        <v>0.0014</v>
+        <v>0.001</v>
       </c>
       <c r="F32" s="71" t="inlineStr">
         <is>
-          <t>→ 0.2%</t>
+          <t>→ 0.3%</t>
         </is>
       </c>
       <c r="G32" s="72" t="inlineStr">
@@ -9756,7 +9756,7 @@
       <c r="E33" s="73" t="n">
         <v>0.001</v>
       </c>
-      <c r="F33" s="77" t="inlineStr">
+      <c r="F33" s="78" t="inlineStr">
         <is>
           <t>↓ 0.6%</t>
         </is>
@@ -9785,7 +9785,7 @@
         <v>0.002</v>
       </c>
       <c r="E34" s="70" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0007000000000000001</v>
       </c>
       <c r="F34" s="71" t="inlineStr">
         <is>
@@ -9897,23 +9897,23 @@
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>Grupo I</t>
+          <t>Grupo J</t>
         </is>
       </c>
       <c r="D38" s="70" t="n">
-        <v>0.0014</v>
+        <v>0.0017</v>
       </c>
       <c r="E38" s="70" t="n">
-        <v>0.0003</v>
+        <v>0.0002</v>
       </c>
       <c r="F38" s="71" t="inlineStr">
         <is>
-          <t>→ 0.1%</t>
+          <t>→ 0.2%</t>
         </is>
       </c>
       <c r="G38" s="72" t="inlineStr">
@@ -9928,23 +9928,23 @@
       </c>
       <c r="B39" s="11" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="C39" s="10" t="inlineStr">
         <is>
-          <t>Grupo J</t>
+          <t>Grupo I</t>
         </is>
       </c>
       <c r="D39" s="73" t="n">
-        <v>0.0017</v>
+        <v>0.0014</v>
       </c>
       <c r="E39" s="73" t="n">
         <v>0.0002</v>
       </c>
       <c r="F39" s="79" t="inlineStr">
         <is>
-          <t>→ 0.2%</t>
+          <t>→ 0.1%</t>
         </is>
       </c>
       <c r="G39" s="75" t="inlineStr">
@@ -10033,7 +10033,7 @@
         <v>0.0003</v>
       </c>
       <c r="E42" s="70" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F42" s="71" t="inlineStr">
         <is>
@@ -10052,19 +10052,19 @@
       </c>
       <c r="B43" s="11" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="C43" s="10" t="inlineStr">
         <is>
-          <t>Grupo A</t>
+          <t>Grupo B</t>
         </is>
       </c>
       <c r="D43" s="73" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="E43" s="73" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F43" s="79" t="inlineStr">
         <is>
@@ -10083,19 +10083,19 @@
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>Grupo B</t>
+          <t>Grupo H</t>
         </is>
       </c>
       <c r="D44" s="70" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="E44" s="70" t="n">
         <v>0</v>
-      </c>
-      <c r="E44" s="70" t="n">
-        <v>0.0001</v>
       </c>
       <c r="F44" s="71" t="inlineStr">
         <is>
@@ -10114,19 +10114,19 @@
       </c>
       <c r="B45" s="11" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C45" s="10" t="inlineStr">
         <is>
-          <t>Grupo H</t>
+          <t>Grupo L</t>
         </is>
       </c>
       <c r="D45" s="73" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="E45" s="73" t="n">
-        <v>0.0001</v>
+        <v>0</v>
       </c>
       <c r="F45" s="79" t="inlineStr">
         <is>
@@ -10145,16 +10145,16 @@
       </c>
       <c r="B46" s="5" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>Grupo E</t>
+          <t>Grupo A</t>
         </is>
       </c>
       <c r="D46" s="70" t="n">
-        <v>0.0001</v>
+        <v>0.0002</v>
       </c>
       <c r="E46" s="70" t="n">
         <v>0</v>
@@ -10176,12 +10176,12 @@
       </c>
       <c r="B47" s="11" t="inlineStr">
         <is>
-          <t>Cape Verde</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C47" s="10" t="inlineStr">
         <is>
-          <t>Grupo H</t>
+          <t>Grupo E</t>
         </is>
       </c>
       <c r="D47" s="73" t="n">
@@ -10207,16 +10207,16 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>Cape Verde</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>Grupo D</t>
+          <t>Grupo H</t>
         </is>
       </c>
       <c r="D48" s="70" t="n">
-        <v>0.0003</v>
+        <v>0.0001</v>
       </c>
       <c r="E48" s="70" t="n">
         <v>0</v>
@@ -10238,16 +10238,16 @@
       </c>
       <c r="B49" s="11" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Haiti</t>
         </is>
       </c>
       <c r="C49" s="10" t="inlineStr">
         <is>
-          <t>Grupo B</t>
+          <t>Grupo D</t>
         </is>
       </c>
       <c r="D49" s="73" t="n">
-        <v>0</v>
+        <v>0.0003</v>
       </c>
       <c r="E49" s="73" t="n">
         <v>0</v>
@@ -10258,37 +10258,6 @@
         </is>
       </c>
       <c r="G49" s="75" t="inlineStr">
-        <is>
-          <t>░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="4" t="n">
-        <v>48</v>
-      </c>
-      <c r="B50" s="5" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="C50" s="4" t="inlineStr">
-        <is>
-          <t>Grupo L</t>
-        </is>
-      </c>
-      <c r="D50" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="E50" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="F50" s="71" t="inlineStr">
-        <is>
-          <t>→ 0.0%</t>
-        </is>
-      </c>
-      <c r="G50" s="72" t="inlineStr">
         <is>
           <t>░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░░</t>
         </is>
@@ -12018,7 +11987,7 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="105" t="inlineStr">
         <is>
-          <t>Brier Score: más bajo = mejor (0 = perfecto, 1 = pésimo). Log-Loss: más bajo = mejor. Naive = 1/n igual prob. a todos. El modelo v2 supera al naive en 9.8% en Brier Score y 53% en Log-Loss (Qatar 2022).</t>
+          <t>Brier Score: más bajo = mejor (0 = perfecto, 1 = pésimo). Log-Loss: más bajo = mejor. Naive = 1/n igual prob. a todos. El modelo v3 supera al naive en 9.8% en Brier Score y 53% en Log-Loss (Qatar 2022).</t>
         </is>
       </c>
     </row>

</xml_diff>